<commit_message>
Fixup on new items; add flag SFL_US;
</commit_message>
<xml_diff>
--- a/src/index spreadsheet/New and updated labels for Chef menu_rj_jm.xlsx
+++ b/src/index spreadsheet/New and updated labels for Chef menu_rj_jm.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jacomostert/wp43s/src/index spreadsheet/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14234EB1-98E8-3E44-B1AF-037F6CB95FDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F69650D8-B696-0746-A9BE-43274DB0E2A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="480" windowWidth="33600" windowHeight="20520" xr2:uid="{95F5296B-734B-A140-B6F4-11B4F81E2566}"/>
+    <workbookView xWindow="5380" yWindow="600" windowWidth="32800" windowHeight="20500" activeTab="2" xr2:uid="{95F5296B-734B-A140-B6F4-11B4F81E2566}"/>
   </bookViews>
   <sheets>
     <sheet name="Items and code" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="472" uniqueCount="230">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="480" uniqueCount="230">
   <si>
     <t>ITM_PINTLQtoML</t>
   </si>
@@ -694,18 +694,9 @@
     <t>IN3</t>
   </si>
   <si>
-    <t xml:space="preserve"> "in" STD_SUP_3 STD_RIGHT_ARROW "m" STD_litre</t>
-  </si>
-  <si>
     <t>"m" STD_litre STD_RIGHT_ARROW "in" STD_SUP_3</t>
   </si>
   <si>
-    <t>"ft" STD_SUP_3 STD_RIGHT_ARROW "GL" STD_UK</t>
-  </si>
-  <si>
-    <t>"GL" STD_UK STD_RIGHT_ARROW "ft" STD_SUP_3</t>
-  </si>
-  <si>
     <t>STD_litre STD_RIGHT_ARROW "ft" STD_SUP_3</t>
   </si>
   <si>
@@ -731,6 +722,15 @@
   </si>
   <si>
     <t>ml x 1000</t>
+  </si>
+  <si>
+    <t>"ft" STD_SUP_3 STD_RIGHT_ARROW "gal" STD_UK</t>
+  </si>
+  <si>
+    <t>"gal" STD_UK STD_RIGHT_ARROW "ft" STD_SUP_3</t>
+  </si>
+  <si>
+    <t>"in" STD_SUP_3 STD_RIGHT_ARROW "m" STD_litre</t>
   </si>
 </sst>
 </file>
@@ -3362,15 +3362,15 @@
         <v>multiply</v>
       </c>
       <c r="F35" s="81" t="str">
-        <f t="shared" ref="F35:F43" si="6" xml:space="preserve"> VLOOKUP(A35,stdform,2,0)</f>
+        <f t="shared" ref="F35:F42" si="6" xml:space="preserve"> VLOOKUP(A35,stdform,2,0)</f>
         <v>"tsp" STD_UK STD_RIGHT_ARROW "ml"</v>
       </c>
       <c r="G35" s="81" t="str">
-        <f t="shared" ref="G35:G43" si="7">MID(F35,1,SEARCH("STD_RIGHT_ARROW",F35)-2)&amp;" STD_RIGHT_ARROW"</f>
+        <f t="shared" ref="G35:G42" si="7">MID(F35,1,SEARCH("STD_RIGHT_ARROW",F35)-2)&amp;" STD_RIGHT_ARROW"</f>
         <v>"tsp" STD_UK STD_RIGHT_ARROW</v>
       </c>
       <c r="H35" s="49" t="str">
-        <f t="shared" ref="H35:H43" si="8">"/* NNNN */  UNIT_CONV("&amp;D35&amp;","&amp;REPT(CHAR(32),21-LEN(D35))&amp;"    "&amp;E35&amp;",      "&amp;F35&amp;","&amp;REPT(CHAR(32),60-LEN(F35))&amp;G35&amp;REPT(CHAR(32),60-LEN(G35))&amp;"),"</f>
+        <f t="shared" ref="H35:H42" si="8">"/* NNNN */  UNIT_CONV("&amp;D35&amp;","&amp;REPT(CHAR(32),21-LEN(D35))&amp;"    "&amp;E35&amp;",      "&amp;F35&amp;","&amp;REPT(CHAR(32),60-LEN(F35))&amp;G35&amp;REPT(CHAR(32),60-LEN(G35))&amp;"),"</f>
         <v>/* NNNN */  UNIT_CONV(constFactorTspukMl,       multiply,      "tsp" STD_UK STD_RIGHT_ARROW "ml",                           "tsp" STD_UK STD_RIGHT_ARROW                                ),</v>
       </c>
       <c r="I35" s="79">
@@ -3378,7 +3378,7 @@
         <v>5.9193880208333001</v>
       </c>
       <c r="J35" s="79" t="str">
-        <f t="shared" ref="J35:J43" si="9">SUBSTITUTE(TEXT(I35,"0.000000000000000000000000000000000000000000000000000000E+00"),"E","e")</f>
+        <f t="shared" ref="J35:J42" si="9">SUBSTITUTE(TEXT(I35,"0.000000000000000000000000000000000000000000000000000000E+00"),"E","e")</f>
         <v>5.919388020833300000000000000000000000000000000000000000e+00</v>
       </c>
       <c r="K35" s="82" t="str">
@@ -3386,11 +3386,11 @@
         <v>TspukMl</v>
       </c>
       <c r="L35" s="50" t="str">
-        <f t="shared" ref="L35:L43" si="10">IF(E35="multiply","  generateConstantArray("&amp;CHAR(34)&amp;K35&amp;CHAR(34)&amp;","&amp;REPT(CHAR(32),14-LEN(K35))&amp;CHAR(34)&amp;"+"&amp;J35&amp;CHAR(34)&amp;");","")</f>
+        <f t="shared" ref="L35:L42" si="10">IF(E35="multiply","  generateConstantArray("&amp;CHAR(34)&amp;K35&amp;CHAR(34)&amp;","&amp;REPT(CHAR(32),14-LEN(K35))&amp;CHAR(34)&amp;"+"&amp;J35&amp;CHAR(34)&amp;");","")</f>
         <v xml:space="preserve">  generateConstantArray("TspukMl",       "+5.919388020833300000000000000000000000000000000000000000e+00");</v>
       </c>
       <c r="N35" s="65" t="str">
-        <f t="shared" ref="N35:N43" si="11">"    ["&amp;D35&amp;"] = "&amp;CHAR(38)&amp;"const_"&amp;K35&amp;","</f>
+        <f t="shared" ref="N35:N42" si="11">"    ["&amp;D35&amp;"] = "&amp;CHAR(38)&amp;"const_"&amp;K35&amp;","</f>
         <v xml:space="preserve">    [constFactorTspukMl] = &amp;const_TspukMl,</v>
       </c>
     </row>
@@ -3465,15 +3465,15 @@
       </c>
       <c r="F37" s="81" t="str">
         <f t="shared" si="6"/>
-        <v xml:space="preserve"> "in" STD_SUP_3 STD_RIGHT_ARROW "m" STD_litre</v>
+        <v>"in" STD_SUP_3 STD_RIGHT_ARROW "m" STD_litre</v>
       </c>
       <c r="G37" s="81" t="str">
         <f t="shared" si="7"/>
-        <v xml:space="preserve"> "in" STD_SUP_3 STD_RIGHT_ARROW</v>
+        <v>"in" STD_SUP_3 STD_RIGHT_ARROW</v>
       </c>
       <c r="H37" s="49" t="str">
         <f t="shared" si="8"/>
-        <v>/* NNNN */  UNIT_CONV(constFactorIn3Ml,         multiply,       "in" STD_SUP_3 STD_RIGHT_ARROW "m" STD_litre,                "in" STD_SUP_3 STD_RIGHT_ARROW                             ),</v>
+        <v>/* NNNN */  UNIT_CONV(constFactorIn3Ml,         multiply,      "in" STD_SUP_3 STD_RIGHT_ARROW "m" STD_litre,                "in" STD_SUP_3 STD_RIGHT_ARROW                              ),</v>
       </c>
       <c r="I37" s="79">
         <f>VLOOKUP(A37,Factors!D:G,4,0)</f>
@@ -3516,7 +3516,7 @@
       </c>
       <c r="F38" s="81" t="str">
         <f t="shared" si="6"/>
-        <v>"ft" STD_SUP_3 STD_RIGHT_ARROW "GL" STD_UK</v>
+        <v>"ft" STD_SUP_3 STD_RIGHT_ARROW "gal" STD_UK</v>
       </c>
       <c r="G38" s="81" t="str">
         <f t="shared" si="7"/>
@@ -3524,7 +3524,7 @@
       </c>
       <c r="H38" s="49" t="str">
         <f t="shared" si="8"/>
-        <v>/* NNNN */  UNIT_CONV(constFactorFt3Gluk,       multiply,      "ft" STD_SUP_3 STD_RIGHT_ARROW "GL" STD_UK,                  "ft" STD_SUP_3 STD_RIGHT_ARROW                              ),</v>
+        <v>/* NNNN */  UNIT_CONV(constFactorFt3Gluk,       multiply,      "ft" STD_SUP_3 STD_RIGHT_ARROW "gal" STD_UK,                 "ft" STD_SUP_3 STD_RIGHT_ARROW                              ),</v>
       </c>
       <c r="I38" s="79">
         <f>VLOOKUP(A38,Factors!D:G,4,0)</f>
@@ -3567,15 +3567,15 @@
       </c>
       <c r="F39" s="81" t="str">
         <f t="shared" si="6"/>
-        <v>"GL" STD_UK STD_RIGHT_ARROW "ft" STD_SUP_3</v>
+        <v>"gal" STD_UK STD_RIGHT_ARROW "ft" STD_SUP_3</v>
       </c>
       <c r="G39" s="81" t="str">
         <f t="shared" si="7"/>
-        <v>"GL" STD_UK STD_RIGHT_ARROW</v>
+        <v>"gal" STD_UK STD_RIGHT_ARROW</v>
       </c>
       <c r="H39" s="49" t="str">
         <f t="shared" si="8"/>
-        <v>/* NNNN */  UNIT_CONV(constFactorGlukFt3,         divide,      "GL" STD_UK STD_RIGHT_ARROW "ft" STD_SUP_3,                  "GL" STD_UK STD_RIGHT_ARROW                                 ),</v>
+        <v>/* NNNN */  UNIT_CONV(constFactorGlukFt3,         divide,      "gal" STD_UK STD_RIGHT_ARROW "ft" STD_SUP_3,                 "gal" STD_UK STD_RIGHT_ARROW                                ),</v>
       </c>
       <c r="I39" s="79">
         <f>VLOOKUP(A39,Factors!D:G,4,0)</f>
@@ -3843,7 +3843,7 @@
     <col min="3" max="3" width="7.83203125" style="7" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="19" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="29" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.83203125" style="8" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="25.5" style="8" customWidth="1"/>
     <col min="7" max="7" width="15.6640625" style="7" bestFit="1" customWidth="1"/>
     <col min="8" max="9" width="16.83203125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="12.33203125" bestFit="1" customWidth="1"/>
@@ -4090,7 +4090,7 @@
     </row>
     <row r="13" spans="1:14" ht="19" thickBot="1">
       <c r="A13" s="77" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="C13" s="27" t="s">
         <v>73</v>
@@ -4111,7 +4111,7 @@
     </row>
     <row r="14" spans="1:14">
       <c r="A14" s="77" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="C14" s="24" t="s">
         <v>76</v>
@@ -4214,34 +4214,34 @@
         <v>16.387063999999999</v>
       </c>
       <c r="G19" s="7" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="J19" s="43"/>
       <c r="K19" s="44"/>
     </row>
     <row r="20" spans="1:14">
       <c r="C20" s="77" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="F20" s="78">
         <f>(12*2.54)^3</f>
         <v>28316.846592000002</v>
       </c>
       <c r="G20" s="7" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="J20" s="43"/>
       <c r="K20" s="44"/>
     </row>
     <row r="21" spans="1:14">
       <c r="C21" s="77" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F21" s="53">
         <v>1000</v>
       </c>
       <c r="G21" s="7" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="J21" s="43"/>
       <c r="K21" s="44"/>
@@ -5968,7 +5968,7 @@
         <v>4.8000063351143778</v>
       </c>
       <c r="H61" s="9">
-        <f t="shared" ref="H60:H67" si="27" xml:space="preserve"> VLOOKUP(B61,units,4,0)</f>
+        <f t="shared" ref="H61:H67" si="27" xml:space="preserve"> VLOOKUP(B61,units,4,0)</f>
         <v>16.387063999999999</v>
       </c>
       <c r="I61" s="9">
@@ -6307,7 +6307,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{12AF49E5-C5CF-EF45-BD21-7588D88F54A2}">
-  <dimension ref="A1:B43"/>
+  <dimension ref="A1:C43"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="18" bestFit="1" customWidth="1"/>
@@ -6562,7 +6562,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="33" spans="1:2">
+    <row r="33" spans="1:3">
       <c r="A33" t="s">
         <v>62</v>
       </c>
@@ -6570,7 +6570,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="34" spans="1:2">
+    <row r="34" spans="1:3">
       <c r="A34" t="s">
         <v>60</v>
       </c>
@@ -6578,68 +6578,92 @@
         <v>175</v>
       </c>
     </row>
-    <row r="36" spans="1:2">
+    <row r="36" spans="1:3" ht="18">
       <c r="A36" t="s">
         <v>200</v>
       </c>
       <c r="B36" t="s">
-        <v>218</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2">
+        <v>217</v>
+      </c>
+      <c r="C36" s="69" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" ht="18">
       <c r="A37" t="s">
         <v>201</v>
       </c>
       <c r="B37" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2">
+        <v>229</v>
+      </c>
+      <c r="C37" s="69" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" ht="18">
       <c r="A38" t="s">
         <v>202</v>
       </c>
       <c r="B38" t="s">
-        <v>219</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2">
+        <v>227</v>
+      </c>
+      <c r="C38" s="69" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" ht="18">
       <c r="A39" t="s">
         <v>203</v>
       </c>
       <c r="B39" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2">
+        <v>228</v>
+      </c>
+      <c r="C39" s="69" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" ht="18">
       <c r="A40" t="s">
         <v>204</v>
       </c>
       <c r="B40" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2">
+        <v>218</v>
+      </c>
+      <c r="C40" s="69" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" ht="18">
       <c r="A41" t="s">
         <v>205</v>
       </c>
       <c r="B41" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="42" spans="1:2">
+        <v>219</v>
+      </c>
+      <c r="C41" s="69" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" ht="18">
       <c r="A42" t="s">
         <v>206</v>
       </c>
       <c r="B42" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="43" spans="1:2">
+        <v>220</v>
+      </c>
+      <c r="C42" s="69" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" ht="18">
       <c r="A43" t="s">
         <v>207</v>
       </c>
       <c r="B43" t="s">
-        <v>224</v>
+        <v>221</v>
+      </c>
+      <c r="C43" s="69" t="s">
+        <v>215</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add floz <> gal
</commit_message>
<xml_diff>
--- a/src/index spreadsheet/New and updated labels for Chef menu_rj_jm.xlsx
+++ b/src/index spreadsheet/New and updated labels for Chef menu_rj_jm.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jacomostert/wp43s/src/index spreadsheet/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C14D795B-DB59-2B4E-9AA5-C58D6E9605F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C17E99C-2B47-CF48-8EA2-F06D21EC4DDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="32780" windowHeight="20500" activeTab="1" xr2:uid="{95F5296B-734B-A140-B6F4-11B4F81E2566}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="525" uniqueCount="262">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="545" uniqueCount="270">
   <si>
     <t>ITM_PINTLQtoML</t>
   </si>
@@ -985,6 +985,30 @@
   <si>
     <t>"ml" STD_RIGHT_ARROW "qt" STD_UK</t>
   </si>
+  <si>
+    <t>ITM_GLUKtoFZUK</t>
+  </si>
+  <si>
+    <t>ITM_FZUKtoGLUK</t>
+  </si>
+  <si>
+    <t>ITM_GLUStoFZUS</t>
+  </si>
+  <si>
+    <t>ITM_FZUStoGLUS</t>
+  </si>
+  <si>
+    <t>"gal" STD_UK STD_RIGHT_ARROW "floz" STD_UK</t>
+  </si>
+  <si>
+    <t>"floz" STD_UK STD_RIGHT_ARROW "gal" STD_UK</t>
+  </si>
+  <si>
+    <t>"gal" STD_US STD_RIGHT_ARROW "floz" STD_US</t>
+  </si>
+  <si>
+    <t>"floz" STD_US STD_RIGHT_ARROW "gal" STD_US</t>
+  </si>
 </sst>
 </file>
 
@@ -998,9 +1022,9 @@
     <numFmt numFmtId="168" formatCode="0.0000000"/>
     <numFmt numFmtId="169" formatCode="0.00000000000"/>
     <numFmt numFmtId="170" formatCode="0.000000000000000"/>
-    <numFmt numFmtId="172" formatCode="0.00000000000000"/>
+    <numFmt numFmtId="171" formatCode="0.00000000000000"/>
   </numFmts>
-  <fonts count="29">
+  <fonts count="32">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1179,8 +1203,27 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color theme="0"/>
+      <name val="C47__StandardFont StandardFont"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="18">
+  <fills count="19">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1280,6 +1323,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1466,7 +1515,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="98">
+  <cellXfs count="101">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
@@ -1580,9 +1629,6 @@
     <xf numFmtId="0" fontId="4" fillId="12" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="12" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="12" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
@@ -1679,7 +1725,7 @@
       <alignment horizontal="left" indent="1"/>
     </xf>
     <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="172" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="166" fontId="10" fillId="17" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -1689,6 +1735,16 @@
     <xf numFmtId="0" fontId="28" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="29" fillId="18" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="18" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="12" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2023,16 +2079,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8086E2D2-A619-CD41-963B-CA5F79ED1F95}">
-  <dimension ref="A1:N46"/>
+  <dimension ref="A1:N50"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="19.5" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16.6640625" style="2" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="5.6640625" customWidth="1"/>
     <col min="4" max="4" width="20.83203125" customWidth="1"/>
-    <col min="5" max="7" width="10.5" style="53" customWidth="1"/>
+    <col min="5" max="7" width="10.5" style="52" customWidth="1"/>
     <col min="8" max="8" width="225" bestFit="1" customWidth="1"/>
-    <col min="9" max="11" width="5.83203125" style="53" customWidth="1"/>
+    <col min="9" max="11" width="5.83203125" style="52" customWidth="1"/>
     <col min="12" max="12" width="144.83203125" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="39.33203125" bestFit="1" customWidth="1"/>
   </cols>
@@ -2040,7 +2096,7 @@
     <row r="1" spans="1:14" ht="16">
       <c r="A1"/>
       <c r="B1"/>
-      <c r="F1" s="53">
+      <c r="F1" s="52">
         <f>LEN(F24)</f>
         <v>57</v>
       </c>
@@ -2065,25 +2121,25 @@
       <c r="D3" s="33" t="s">
         <v>183</v>
       </c>
-      <c r="E3" s="54" t="s">
+      <c r="E3" s="53" t="s">
         <v>184</v>
       </c>
-      <c r="F3" s="54" t="s">
+      <c r="F3" s="53" t="s">
         <v>184</v>
       </c>
-      <c r="G3" s="54" t="s">
+      <c r="G3" s="53" t="s">
         <v>184</v>
       </c>
       <c r="H3" s="33" t="s">
         <v>181</v>
       </c>
-      <c r="I3" s="54" t="s">
+      <c r="I3" s="53" t="s">
         <v>184</v>
       </c>
-      <c r="J3" s="54" t="s">
+      <c r="J3" s="53" t="s">
         <v>184</v>
       </c>
-      <c r="K3" s="54" t="s">
+      <c r="K3" s="53" t="s">
         <v>184</v>
       </c>
       <c r="L3" s="33" t="s">
@@ -2100,22 +2156,22 @@
       <c r="B4" s="43" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="91" t="s">
+      <c r="C4" s="90" t="s">
         <v>70</v>
       </c>
       <c r="D4" s="40" t="str">
         <f>VLOOKUP(A4,Factors!D:K,8,0)</f>
         <v>constFactorCupcFzus</v>
       </c>
-      <c r="E4" s="53" t="str">
+      <c r="E4" s="52" t="str">
         <f>VLOOKUP(A4,Factors!D:N,10,0)</f>
         <v>multiply</v>
       </c>
-      <c r="F4" s="55" t="str">
-        <f t="shared" ref="F4:F43" si="0" xml:space="preserve"> VLOOKUP(A4,stdform,2,0)</f>
+      <c r="F4" s="54" t="str">
+        <f t="shared" ref="F4:F47" si="0" xml:space="preserve"> VLOOKUP(A4,stdform,2,0)</f>
         <v>"cup" STD_US STD_SUB_c STD_RIGHT_ARROW "floz" STD_US</v>
       </c>
-      <c r="G4" s="55" t="str">
+      <c r="G4" s="54" t="str">
         <f>MID(F4,1,SEARCH("STD_RIGHT_ARROW",F4)-2)&amp;" STD_RIGHT_ARROW"</f>
         <v>"cup" STD_US STD_SUB_c STD_RIGHT_ARROW</v>
       </c>
@@ -2123,15 +2179,15 @@
         <f>"/* NNNN */  UNIT_CONV("&amp;D4&amp;","&amp;REPT(CHAR(32),21-LEN(D4))&amp;"    "&amp;E4&amp;",      "&amp;F4&amp;","&amp;REPT(CHAR(32),60-LEN(F4))&amp;G4&amp;REPT(CHAR(32),60-LEN(G4))&amp;"),"</f>
         <v>/* NNNN */  UNIT_CONV(constFactorCupcFzus,      multiply,      "cup" STD_US STD_SUB_c STD_RIGHT_ARROW "floz" STD_US,        "cup" STD_US STD_SUB_c STD_RIGHT_ARROW                      ),</v>
       </c>
-      <c r="I4" s="56">
+      <c r="I4" s="55">
         <f>VLOOKUP(A4,Factors!D:G,4,0)</f>
         <v>8</v>
       </c>
-      <c r="J4" s="53" t="str">
+      <c r="J4" s="52" t="str">
         <f>SUBSTITUTE(TEXT(I4,"0.000000000000000000000000000000000000000000000000000000E+00"),"E","e")</f>
         <v>8.000000000000000000000000000000000000000000000000000000e+00</v>
       </c>
-      <c r="K4" s="56" t="str">
+      <c r="K4" s="55" t="str">
         <f>VLOOKUP(A4,Factors!D:N,11,0)</f>
         <v>CupcFzus</v>
       </c>
@@ -2151,47 +2207,47 @@
       <c r="B5" s="43" t="s">
         <v>19</v>
       </c>
-      <c r="C5" s="91" t="s">
+      <c r="C5" s="90" t="s">
         <v>70</v>
       </c>
       <c r="D5" s="40" t="str">
         <f>VLOOKUP(A5,Factors!D:K,8,0)</f>
         <v>constFactorCupcMl</v>
       </c>
-      <c r="E5" s="53" t="str">
+      <c r="E5" s="52" t="str">
         <f>VLOOKUP(A5,Factors!D:N,10,0)</f>
         <v>multiply</v>
       </c>
-      <c r="F5" s="55" t="str">
+      <c r="F5" s="54" t="str">
         <f t="shared" si="0"/>
         <v>"cup" STD_US STD_SUB_c STD_RIGHT_ARROW "ml"</v>
       </c>
-      <c r="G5" s="55" t="str">
-        <f t="shared" ref="G5:G43" si="1">MID(F5,1,SEARCH("STD_RIGHT_ARROW",F5)-2)&amp;" STD_RIGHT_ARROW"</f>
+      <c r="G5" s="54" t="str">
+        <f t="shared" ref="G5:G47" si="1">MID(F5,1,SEARCH("STD_RIGHT_ARROW",F5)-2)&amp;" STD_RIGHT_ARROW"</f>
         <v>"cup" STD_US STD_SUB_c STD_RIGHT_ARROW</v>
       </c>
       <c r="H5" s="30" t="str">
-        <f t="shared" ref="H5:H43" si="2">"/* NNNN */  UNIT_CONV("&amp;D5&amp;","&amp;REPT(CHAR(32),21-LEN(D5))&amp;"    "&amp;E5&amp;",      "&amp;F5&amp;","&amp;REPT(CHAR(32),60-LEN(F5))&amp;G5&amp;REPT(CHAR(32),60-LEN(G5))&amp;"),"</f>
+        <f t="shared" ref="H5:H47" si="2">"/* NNNN */  UNIT_CONV("&amp;D5&amp;","&amp;REPT(CHAR(32),21-LEN(D5))&amp;"    "&amp;E5&amp;",      "&amp;F5&amp;","&amp;REPT(CHAR(32),60-LEN(F5))&amp;G5&amp;REPT(CHAR(32),60-LEN(G5))&amp;"),"</f>
         <v>/* NNNN */  UNIT_CONV(constFactorCupcMl,        multiply,      "cup" STD_US STD_SUB_c STD_RIGHT_ARROW "ml",                 "cup" STD_US STD_SUB_c STD_RIGHT_ARROW                      ),</v>
       </c>
-      <c r="I5" s="53">
+      <c r="I5" s="52">
         <f>VLOOKUP(A5,Factors!D:G,4,0)</f>
         <v>236.58823649999999</v>
       </c>
-      <c r="J5" s="53" t="str">
-        <f t="shared" ref="J5:J43" si="3">SUBSTITUTE(TEXT(I5,"0.000000000000000000000000000000000000000000000000000000E+00"),"E","e")</f>
+      <c r="J5" s="52" t="str">
+        <f t="shared" ref="J5:J47" si="3">SUBSTITUTE(TEXT(I5,"0.000000000000000000000000000000000000000000000000000000E+00"),"E","e")</f>
         <v>2.365882365000000000000000000000000000000000000000000000e+02</v>
       </c>
-      <c r="K5" s="56" t="str">
+      <c r="K5" s="55" t="str">
         <f>VLOOKUP(A5,Factors!D:N,11,0)</f>
         <v>CupcMl</v>
       </c>
       <c r="L5" s="31" t="str">
-        <f t="shared" ref="L5:L43" si="4">IF(E5="multiply","  generateConstantArray("&amp;CHAR(34)&amp;K5&amp;CHAR(34)&amp;","&amp;REPT(CHAR(32),14-LEN(K5))&amp;CHAR(34)&amp;"+"&amp;J5&amp;CHAR(34)&amp;");","")</f>
+        <f t="shared" ref="L5:L47" si="4">IF(E5="multiply","  generateConstantArray("&amp;CHAR(34)&amp;K5&amp;CHAR(34)&amp;","&amp;REPT(CHAR(32),14-LEN(K5))&amp;CHAR(34)&amp;"+"&amp;J5&amp;CHAR(34)&amp;");","")</f>
         <v xml:space="preserve">  generateConstantArray("CupcMl",        "+2.365882365000000000000000000000000000000000000000000000e+02");</v>
       </c>
       <c r="N5" s="41" t="str">
-        <f t="shared" ref="N5:N43" si="5">"    ["&amp;D5&amp;"] = "&amp;CHAR(38)&amp;"const_"&amp;K5&amp;","</f>
+        <f t="shared" ref="N5:N47" si="5">"    ["&amp;D5&amp;"] = "&amp;CHAR(38)&amp;"const_"&amp;K5&amp;","</f>
         <v xml:space="preserve">    [constFactorCupcMl] = &amp;const_CupcMl,</v>
       </c>
     </row>
@@ -2202,22 +2258,22 @@
       <c r="B6" s="43" t="s">
         <v>39</v>
       </c>
-      <c r="C6" s="91" t="s">
+      <c r="C6" s="90" t="s">
         <v>70</v>
       </c>
       <c r="D6" s="40" t="str">
         <f>VLOOKUP(A6,Factors!D:K,8,0)</f>
         <v>constFactorCupukFzuk</v>
       </c>
-      <c r="E6" s="53" t="str">
+      <c r="E6" s="52" t="str">
         <f>VLOOKUP(A6,Factors!D:N,10,0)</f>
         <v>multiply</v>
       </c>
-      <c r="F6" s="55" t="str">
+      <c r="F6" s="54" t="str">
         <f t="shared" si="0"/>
         <v>"cup" STD_UK STD_RIGHT_ARROW "floz" STD_UK</v>
       </c>
-      <c r="G6" s="55" t="str">
+      <c r="G6" s="54" t="str">
         <f t="shared" si="1"/>
         <v>"cup" STD_UK STD_RIGHT_ARROW</v>
       </c>
@@ -2225,15 +2281,15 @@
         <f t="shared" si="2"/>
         <v>/* NNNN */  UNIT_CONV(constFactorCupukFzuk,     multiply,      "cup" STD_UK STD_RIGHT_ARROW "floz" STD_UK,                  "cup" STD_UK STD_RIGHT_ARROW                                ),</v>
       </c>
-      <c r="I6" s="53">
+      <c r="I6" s="52">
         <f>VLOOKUP(A6,Factors!D:G,4,0)</f>
         <v>10</v>
       </c>
-      <c r="J6" s="53" t="str">
+      <c r="J6" s="52" t="str">
         <f t="shared" si="3"/>
         <v>1.000000000000000000000000000000000000000000000000000000e+01</v>
       </c>
-      <c r="K6" s="56" t="str">
+      <c r="K6" s="55" t="str">
         <f>VLOOKUP(A6,Factors!D:N,11,0)</f>
         <v>CupukFzuk</v>
       </c>
@@ -2253,22 +2309,22 @@
       <c r="B7" s="43" t="s">
         <v>47</v>
       </c>
-      <c r="C7" s="91" t="s">
+      <c r="C7" s="90" t="s">
         <v>70</v>
       </c>
       <c r="D7" s="40" t="str">
         <f>VLOOKUP(A7,Factors!D:K,8,0)</f>
         <v>constFactorCupukMl</v>
       </c>
-      <c r="E7" s="53" t="str">
+      <c r="E7" s="52" t="str">
         <f>VLOOKUP(A7,Factors!D:N,10,0)</f>
         <v>multiply</v>
       </c>
-      <c r="F7" s="55" t="str">
+      <c r="F7" s="54" t="str">
         <f t="shared" si="0"/>
         <v>"cup" STD_UK STD_RIGHT_ARROW "ml"</v>
       </c>
-      <c r="G7" s="55" t="str">
+      <c r="G7" s="54" t="str">
         <f t="shared" si="1"/>
         <v>"cup" STD_UK STD_RIGHT_ARROW</v>
       </c>
@@ -2276,15 +2332,15 @@
         <f t="shared" si="2"/>
         <v>/* NNNN */  UNIT_CONV(constFactorCupukMl,       multiply,      "cup" STD_UK STD_RIGHT_ARROW "ml",                           "cup" STD_UK STD_RIGHT_ARROW                                ),</v>
       </c>
-      <c r="I7" s="53">
+      <c r="I7" s="52">
         <f>VLOOKUP(A7,Factors!D:G,4,0)</f>
         <v>284.13062500000001</v>
       </c>
-      <c r="J7" s="53" t="str">
+      <c r="J7" s="52" t="str">
         <f t="shared" si="3"/>
         <v>2.841306250000000000000000000000000000000000000000000000e+02</v>
       </c>
-      <c r="K7" s="56" t="str">
+      <c r="K7" s="55" t="str">
         <f>VLOOKUP(A7,Factors!D:N,11,0)</f>
         <v>CupukMl</v>
       </c>
@@ -2304,22 +2360,22 @@
       <c r="B8" s="43" t="s">
         <v>37</v>
       </c>
-      <c r="C8" s="91" t="s">
+      <c r="C8" s="90" t="s">
         <v>70</v>
       </c>
       <c r="D8" s="40" t="str">
         <f>VLOOKUP(A8,Factors!D:K,8,0)</f>
         <v>constFactorFzukCupuk</v>
       </c>
-      <c r="E8" s="53" t="str">
+      <c r="E8" s="52" t="str">
         <f>VLOOKUP(A8,Factors!D:N,10,0)</f>
         <v xml:space="preserve">  divide</v>
       </c>
-      <c r="F8" s="55" t="str">
+      <c r="F8" s="54" t="str">
         <f t="shared" si="0"/>
         <v>"floz" STD_UK STD_RIGHT_ARROW "cup" STD_UK</v>
       </c>
-      <c r="G8" s="55" t="str">
+      <c r="G8" s="54" t="str">
         <f t="shared" si="1"/>
         <v>"floz" STD_UK STD_RIGHT_ARROW</v>
       </c>
@@ -2327,15 +2383,15 @@
         <f t="shared" si="2"/>
         <v>/* NNNN */  UNIT_CONV(constFactorFzukCupuk,       divide,      "floz" STD_UK STD_RIGHT_ARROW "cup" STD_UK,                  "floz" STD_UK STD_RIGHT_ARROW                               ),</v>
       </c>
-      <c r="I8" s="53">
+      <c r="I8" s="52">
         <f>VLOOKUP(A8,Factors!D:G,4,0)</f>
         <v>10</v>
       </c>
-      <c r="J8" s="53" t="str">
+      <c r="J8" s="52" t="str">
         <f t="shared" si="3"/>
         <v>1.000000000000000000000000000000000000000000000000000000e+01</v>
       </c>
-      <c r="K8" s="56" t="str">
+      <c r="K8" s="55" t="str">
         <f>VLOOKUP(A8,Factors!D:N,11,0)</f>
         <v>CupukFzuk</v>
       </c>
@@ -2355,22 +2411,22 @@
       <c r="B9" s="43" t="s">
         <v>41</v>
       </c>
-      <c r="C9" s="91" t="s">
+      <c r="C9" s="90" t="s">
         <v>70</v>
       </c>
       <c r="D9" s="40" t="str">
         <f>VLOOKUP(A9,Factors!D:K,8,0)</f>
         <v>constFactorFzukTbspuk</v>
       </c>
-      <c r="E9" s="53" t="str">
+      <c r="E9" s="52" t="str">
         <f>VLOOKUP(A9,Factors!D:N,10,0)</f>
         <v>multiply</v>
       </c>
-      <c r="F9" s="55" t="str">
+      <c r="F9" s="54" t="str">
         <f t="shared" si="0"/>
         <v>"floz" STD_UK STD_RIGHT_ARROW "Tbsp" STD_UK</v>
       </c>
-      <c r="G9" s="55" t="str">
+      <c r="G9" s="54" t="str">
         <f t="shared" si="1"/>
         <v>"floz" STD_UK STD_RIGHT_ARROW</v>
       </c>
@@ -2378,15 +2434,15 @@
         <f t="shared" si="2"/>
         <v>/* NNNN */  UNIT_CONV(constFactorFzukTbspuk,    multiply,      "floz" STD_UK STD_RIGHT_ARROW "Tbsp" STD_UK,                 "floz" STD_UK STD_RIGHT_ARROW                               ),</v>
       </c>
-      <c r="I9" s="53">
+      <c r="I9" s="52">
         <f>VLOOKUP(A9,Factors!D:G,4,0)</f>
         <v>1.6</v>
       </c>
-      <c r="J9" s="53" t="str">
+      <c r="J9" s="52" t="str">
         <f t="shared" si="3"/>
         <v>1.600000000000000000000000000000000000000000000000000000e+00</v>
       </c>
-      <c r="K9" s="56" t="str">
+      <c r="K9" s="55" t="str">
         <f>VLOOKUP(A9,Factors!D:N,11,0)</f>
         <v>FzukTbspuk</v>
       </c>
@@ -2406,22 +2462,22 @@
       <c r="B10" s="43" t="s">
         <v>63</v>
       </c>
-      <c r="C10" s="91" t="s">
+      <c r="C10" s="90" t="s">
         <v>70</v>
       </c>
       <c r="D10" s="40" t="str">
         <f>VLOOKUP(A10,Factors!D:K,8,0)</f>
         <v>constFactorFzukTspuk</v>
       </c>
-      <c r="E10" s="53" t="str">
+      <c r="E10" s="52" t="str">
         <f>VLOOKUP(A10,Factors!D:N,10,0)</f>
         <v>multiply</v>
       </c>
-      <c r="F10" s="55" t="str">
+      <c r="F10" s="54" t="str">
         <f t="shared" si="0"/>
         <v>"floz" STD_UK STD_RIGHT_ARROW "tsp" STD_UK</v>
       </c>
-      <c r="G10" s="55" t="str">
+      <c r="G10" s="54" t="str">
         <f t="shared" si="1"/>
         <v>"floz" STD_UK STD_RIGHT_ARROW</v>
       </c>
@@ -2429,15 +2485,15 @@
         <f t="shared" si="2"/>
         <v>/* NNNN */  UNIT_CONV(constFactorFzukTspuk,     multiply,      "floz" STD_UK STD_RIGHT_ARROW "tsp" STD_UK,                  "floz" STD_UK STD_RIGHT_ARROW                               ),</v>
       </c>
-      <c r="I10" s="53">
+      <c r="I10" s="52">
         <f>VLOOKUP(A10,Factors!D:G,4,0)</f>
         <v>4.8</v>
       </c>
-      <c r="J10" s="53" t="str">
+      <c r="J10" s="52" t="str">
         <f t="shared" si="3"/>
         <v>4.800000000000000000000000000000000000000000000000000000e+00</v>
       </c>
-      <c r="K10" s="56" t="str">
+      <c r="K10" s="55" t="str">
         <f>VLOOKUP(A10,Factors!D:N,11,0)</f>
         <v>FzukTspuk</v>
       </c>
@@ -2457,22 +2513,22 @@
       <c r="B11" s="43" t="s">
         <v>9</v>
       </c>
-      <c r="C11" s="91" t="s">
+      <c r="C11" s="90" t="s">
         <v>70</v>
       </c>
       <c r="D11" s="40" t="str">
         <f>VLOOKUP(A11,Factors!D:K,8,0)</f>
         <v>constFactorFzusCupc</v>
       </c>
-      <c r="E11" s="53" t="str">
+      <c r="E11" s="52" t="str">
         <f>VLOOKUP(A11,Factors!D:N,10,0)</f>
         <v xml:space="preserve">  divide</v>
       </c>
-      <c r="F11" s="55" t="str">
+      <c r="F11" s="54" t="str">
         <f t="shared" si="0"/>
         <v>"floz" STD_US STD_RIGHT_ARROW "cup" STD_US STD_SUB_c</v>
       </c>
-      <c r="G11" s="55" t="str">
+      <c r="G11" s="54" t="str">
         <f t="shared" si="1"/>
         <v>"floz" STD_US STD_RIGHT_ARROW</v>
       </c>
@@ -2480,15 +2536,15 @@
         <f t="shared" si="2"/>
         <v>/* NNNN */  UNIT_CONV(constFactorFzusCupc,        divide,      "floz" STD_US STD_RIGHT_ARROW "cup" STD_US STD_SUB_c,        "floz" STD_US STD_RIGHT_ARROW                               ),</v>
       </c>
-      <c r="I11" s="53">
+      <c r="I11" s="52">
         <f>VLOOKUP(A11,Factors!D:G,4,0)</f>
         <v>8</v>
       </c>
-      <c r="J11" s="53" t="str">
+      <c r="J11" s="52" t="str">
         <f t="shared" si="3"/>
         <v>8.000000000000000000000000000000000000000000000000000000e+00</v>
       </c>
-      <c r="K11" s="56" t="str">
+      <c r="K11" s="55" t="str">
         <f>VLOOKUP(A11,Factors!D:N,11,0)</f>
         <v>CupcFzus</v>
       </c>
@@ -2508,22 +2564,22 @@
       <c r="B12" s="43" t="s">
         <v>13</v>
       </c>
-      <c r="C12" s="91" t="s">
+      <c r="C12" s="90" t="s">
         <v>70</v>
       </c>
       <c r="D12" s="40" t="str">
         <f>VLOOKUP(A12,Factors!D:K,8,0)</f>
         <v>constFactorFzusTbspc</v>
       </c>
-      <c r="E12" s="53" t="str">
+      <c r="E12" s="52" t="str">
         <f>VLOOKUP(A12,Factors!D:N,10,0)</f>
         <v>multiply</v>
       </c>
-      <c r="F12" s="55" t="str">
+      <c r="F12" s="54" t="str">
         <f t="shared" si="0"/>
         <v>"floz" STD_US STD_RIGHT_ARROW "Tbsp" STD_US STD_SUB_c</v>
       </c>
-      <c r="G12" s="55" t="str">
+      <c r="G12" s="54" t="str">
         <f t="shared" si="1"/>
         <v>"floz" STD_US STD_RIGHT_ARROW</v>
       </c>
@@ -2531,15 +2587,15 @@
         <f t="shared" si="2"/>
         <v>/* NNNN */  UNIT_CONV(constFactorFzusTbspc,     multiply,      "floz" STD_US STD_RIGHT_ARROW "Tbsp" STD_US STD_SUB_c,       "floz" STD_US STD_RIGHT_ARROW                               ),</v>
       </c>
-      <c r="I12" s="53">
+      <c r="I12" s="52">
         <f>VLOOKUP(A12,Factors!D:G,4,0)</f>
         <v>2</v>
       </c>
-      <c r="J12" s="53" t="str">
+      <c r="J12" s="52" t="str">
         <f t="shared" si="3"/>
         <v>2.000000000000000000000000000000000000000000000000000000e+00</v>
       </c>
-      <c r="K12" s="56" t="str">
+      <c r="K12" s="55" t="str">
         <f>VLOOKUP(A12,Factors!D:N,11,0)</f>
         <v>FzusTbspc</v>
       </c>
@@ -2559,22 +2615,22 @@
       <c r="B13" s="43" t="s">
         <v>57</v>
       </c>
-      <c r="C13" s="91" t="s">
+      <c r="C13" s="90" t="s">
         <v>70</v>
       </c>
       <c r="D13" s="40" t="str">
         <f>VLOOKUP(A13,Factors!D:K,8,0)</f>
         <v>constFactorFzusTspc</v>
       </c>
-      <c r="E13" s="53" t="str">
+      <c r="E13" s="52" t="str">
         <f>VLOOKUP(A13,Factors!D:N,10,0)</f>
         <v>multiply</v>
       </c>
-      <c r="F13" s="55" t="str">
+      <c r="F13" s="54" t="str">
         <f t="shared" si="0"/>
         <v>"floz" STD_US STD_RIGHT_ARROW "tsp" STD_US STD_SUB_c</v>
       </c>
-      <c r="G13" s="55" t="str">
+      <c r="G13" s="54" t="str">
         <f t="shared" si="1"/>
         <v>"floz" STD_US STD_RIGHT_ARROW</v>
       </c>
@@ -2582,15 +2638,15 @@
         <f t="shared" si="2"/>
         <v>/* NNNN */  UNIT_CONV(constFactorFzusTspc,      multiply,      "floz" STD_US STD_RIGHT_ARROW "tsp" STD_US STD_SUB_c,        "floz" STD_US STD_RIGHT_ARROW                               ),</v>
       </c>
-      <c r="I13" s="53">
+      <c r="I13" s="52">
         <f>VLOOKUP(A13,Factors!D:G,4,0)</f>
         <v>6</v>
       </c>
-      <c r="J13" s="53" t="str">
+      <c r="J13" s="52" t="str">
         <f t="shared" si="3"/>
         <v>6.000000000000000000000000000000000000000000000000000000e+00</v>
       </c>
-      <c r="K13" s="56" t="str">
+      <c r="K13" s="55" t="str">
         <f>VLOOKUP(A13,Factors!D:N,11,0)</f>
         <v>FzusTspc</v>
       </c>
@@ -2610,22 +2666,22 @@
       <c r="B14" s="43" t="s">
         <v>17</v>
       </c>
-      <c r="C14" s="91" t="s">
+      <c r="C14" s="90" t="s">
         <v>70</v>
       </c>
       <c r="D14" s="40" t="str">
         <f>VLOOKUP(A14,Factors!D:K,8,0)</f>
         <v>constFactorMlCupc</v>
       </c>
-      <c r="E14" s="53" t="str">
+      <c r="E14" s="52" t="str">
         <f>VLOOKUP(A14,Factors!D:N,10,0)</f>
         <v xml:space="preserve">  divide</v>
       </c>
-      <c r="F14" s="55" t="str">
+      <c r="F14" s="54" t="str">
         <f t="shared" si="0"/>
         <v>"ml" STD_RIGHT_ARROW "cup" STD_US STD_SUB_c</v>
       </c>
-      <c r="G14" s="55" t="str">
+      <c r="G14" s="54" t="str">
         <f t="shared" si="1"/>
         <v>"ml" STD_RIGHT_ARROW</v>
       </c>
@@ -2633,15 +2689,15 @@
         <f t="shared" si="2"/>
         <v>/* NNNN */  UNIT_CONV(constFactorMlCupc,          divide,      "ml" STD_RIGHT_ARROW "cup" STD_US STD_SUB_c,                 "ml" STD_RIGHT_ARROW                                        ),</v>
       </c>
-      <c r="I14" s="53">
+      <c r="I14" s="52">
         <f>VLOOKUP(A14,Factors!D:G,4,0)</f>
         <v>236.58823649999999</v>
       </c>
-      <c r="J14" s="53" t="str">
+      <c r="J14" s="52" t="str">
         <f t="shared" si="3"/>
         <v>2.365882365000000000000000000000000000000000000000000000e+02</v>
       </c>
-      <c r="K14" s="56" t="str">
+      <c r="K14" s="55" t="str">
         <f>VLOOKUP(A14,Factors!D:N,11,0)</f>
         <v>CupcMl</v>
       </c>
@@ -2661,22 +2717,22 @@
       <c r="B15" s="43" t="s">
         <v>45</v>
       </c>
-      <c r="C15" s="91" t="s">
+      <c r="C15" s="90" t="s">
         <v>70</v>
       </c>
       <c r="D15" s="40" t="str">
         <f>VLOOKUP(A15,Factors!D:K,8,0)</f>
         <v>constFactorMlCupuk</v>
       </c>
-      <c r="E15" s="53" t="str">
+      <c r="E15" s="52" t="str">
         <f>VLOOKUP(A15,Factors!D:N,10,0)</f>
         <v xml:space="preserve">  divide</v>
       </c>
-      <c r="F15" s="55" t="str">
+      <c r="F15" s="54" t="str">
         <f t="shared" si="0"/>
         <v>"ml" STD_RIGHT_ARROW "cup" STD_UK</v>
       </c>
-      <c r="G15" s="55" t="str">
+      <c r="G15" s="54" t="str">
         <f t="shared" si="1"/>
         <v>"ml" STD_RIGHT_ARROW</v>
       </c>
@@ -2684,15 +2740,15 @@
         <f t="shared" si="2"/>
         <v>/* NNNN */  UNIT_CONV(constFactorMlCupuk,         divide,      "ml" STD_RIGHT_ARROW "cup" STD_UK,                           "ml" STD_RIGHT_ARROW                                        ),</v>
       </c>
-      <c r="I15" s="53">
+      <c r="I15" s="52">
         <f>VLOOKUP(A15,Factors!D:G,4,0)</f>
         <v>284.13062500000001</v>
       </c>
-      <c r="J15" s="53" t="str">
+      <c r="J15" s="52" t="str">
         <f t="shared" si="3"/>
         <v>2.841306250000000000000000000000000000000000000000000000e+02</v>
       </c>
-      <c r="K15" s="56" t="str">
+      <c r="K15" s="55" t="str">
         <f>VLOOKUP(A15,Factors!D:N,11,0)</f>
         <v>CupukMl</v>
       </c>
@@ -2712,22 +2768,22 @@
       <c r="B16" s="43" t="s">
         <v>3</v>
       </c>
-      <c r="C16" s="91" t="s">
+      <c r="C16" s="90" t="s">
         <v>70</v>
       </c>
       <c r="D16" s="40" t="str">
         <f>VLOOKUP(A16,Factors!D:K,8,0)</f>
         <v>constFactorMlPintlq</v>
       </c>
-      <c r="E16" s="53" t="str">
+      <c r="E16" s="52" t="str">
         <f>VLOOKUP(A16,Factors!D:N,10,0)</f>
         <v xml:space="preserve">  divide</v>
       </c>
-      <c r="F16" s="55" t="str">
+      <c r="F16" s="54" t="str">
         <f t="shared" si="0"/>
         <v>"ml" STD_RIGHT_ARROW "pint" STD_SUB_l STD_SUB_i STD_SUB_q</v>
       </c>
-      <c r="G16" s="55" t="str">
+      <c r="G16" s="54" t="str">
         <f t="shared" si="1"/>
         <v>"ml" STD_RIGHT_ARROW</v>
       </c>
@@ -2735,15 +2791,15 @@
         <f t="shared" si="2"/>
         <v>/* NNNN */  UNIT_CONV(constFactorMlPintlq,        divide,      "ml" STD_RIGHT_ARROW "pint" STD_SUB_l STD_SUB_i STD_SUB_q,   "ml" STD_RIGHT_ARROW                                        ),</v>
       </c>
-      <c r="I16" s="53">
+      <c r="I16" s="52">
         <f>VLOOKUP(A16,Factors!D:G,4,0)</f>
         <v>473.17647299999999</v>
       </c>
-      <c r="J16" s="53" t="str">
+      <c r="J16" s="52" t="str">
         <f t="shared" si="3"/>
         <v>4.731764730000000000000000000000000000000000000000000000e+02</v>
       </c>
-      <c r="K16" s="56" t="str">
+      <c r="K16" s="55" t="str">
         <f>VLOOKUP(A16,Factors!D:N,11,0)</f>
         <v>PintlqMl</v>
       </c>
@@ -2763,22 +2819,22 @@
       <c r="B17" s="43" t="s">
         <v>31</v>
       </c>
-      <c r="C17" s="91" t="s">
+      <c r="C17" s="90" t="s">
         <v>70</v>
       </c>
       <c r="D17" s="40" t="str">
         <f>VLOOKUP(A17,Factors!D:K,8,0)</f>
         <v>constFactorMlPintuk</v>
       </c>
-      <c r="E17" s="53" t="str">
+      <c r="E17" s="52" t="str">
         <f>VLOOKUP(A17,Factors!D:N,10,0)</f>
         <v xml:space="preserve">  divide</v>
       </c>
-      <c r="F17" s="55" t="str">
+      <c r="F17" s="54" t="str">
         <f t="shared" si="0"/>
         <v>"ml" STD_RIGHT_ARROW "pint" STD_UK</v>
       </c>
-      <c r="G17" s="55" t="str">
+      <c r="G17" s="54" t="str">
         <f t="shared" si="1"/>
         <v>"ml" STD_RIGHT_ARROW</v>
       </c>
@@ -2786,15 +2842,15 @@
         <f t="shared" si="2"/>
         <v>/* NNNN */  UNIT_CONV(constFactorMlPintuk,        divide,      "ml" STD_RIGHT_ARROW "pint" STD_UK,                          "ml" STD_RIGHT_ARROW                                        ),</v>
       </c>
-      <c r="I17" s="53">
+      <c r="I17" s="52">
         <f>VLOOKUP(A17,Factors!D:G,4,0)</f>
         <v>568.26125000000002</v>
       </c>
-      <c r="J17" s="53" t="str">
+      <c r="J17" s="52" t="str">
         <f t="shared" si="3"/>
         <v>5.682612500000000000000000000000000000000000000000000000e+02</v>
       </c>
-      <c r="K17" s="56" t="str">
+      <c r="K17" s="55" t="str">
         <f>VLOOKUP(A17,Factors!D:N,11,0)</f>
         <v>PintukMl</v>
       </c>
@@ -2814,22 +2870,22 @@
       <c r="B18" s="43" t="s">
         <v>35</v>
       </c>
-      <c r="C18" s="91" t="s">
+      <c r="C18" s="90" t="s">
         <v>70</v>
       </c>
       <c r="D18" s="40" t="str">
         <f>VLOOKUP(A18,Factors!D:K,8,0)</f>
         <v>constFactorMlQt</v>
       </c>
-      <c r="E18" s="53" t="str">
+      <c r="E18" s="52" t="str">
         <f>VLOOKUP(A18,Factors!D:N,10,0)</f>
         <v xml:space="preserve">  divide</v>
       </c>
-      <c r="F18" s="55" t="str">
+      <c r="F18" s="54" t="str">
         <f t="shared" si="0"/>
         <v>"ml" STD_RIGHT_ARROW "qt" STD_UK</v>
       </c>
-      <c r="G18" s="55" t="str">
+      <c r="G18" s="54" t="str">
         <f t="shared" si="1"/>
         <v>"ml" STD_RIGHT_ARROW</v>
       </c>
@@ -2837,15 +2893,15 @@
         <f t="shared" si="2"/>
         <v>/* NNNN */  UNIT_CONV(constFactorMlQt,            divide,      "ml" STD_RIGHT_ARROW "qt" STD_UK,                            "ml" STD_RIGHT_ARROW                                        ),</v>
       </c>
-      <c r="I18" s="53">
+      <c r="I18" s="52">
         <f>VLOOKUP(A18,Factors!D:G,4,0)</f>
         <v>1136.5225</v>
       </c>
-      <c r="J18" s="53" t="str">
+      <c r="J18" s="52" t="str">
         <f t="shared" si="3"/>
         <v>1.136522500000000000000000000000000000000000000000000000e+03</v>
       </c>
-      <c r="K18" s="56" t="str">
+      <c r="K18" s="55" t="str">
         <f>VLOOKUP(A18,Factors!D:N,11,0)</f>
         <v>QtMl</v>
       </c>
@@ -2865,22 +2921,22 @@
       <c r="B19" s="43" t="s">
         <v>7</v>
       </c>
-      <c r="C19" s="91" t="s">
+      <c r="C19" s="90" t="s">
         <v>70</v>
       </c>
       <c r="D19" s="40" t="str">
         <f>VLOOKUP(A19,Factors!D:K,8,0)</f>
         <v>constFactorMlQtus</v>
       </c>
-      <c r="E19" s="53" t="str">
+      <c r="E19" s="52" t="str">
         <f>VLOOKUP(A19,Factors!D:N,10,0)</f>
         <v xml:space="preserve">  divide</v>
       </c>
-      <c r="F19" s="55" t="str">
+      <c r="F19" s="54" t="str">
         <f t="shared" si="0"/>
         <v>"ml" STD_RIGHT_ARROW "qt" STD_US</v>
       </c>
-      <c r="G19" s="55" t="str">
+      <c r="G19" s="54" t="str">
         <f t="shared" si="1"/>
         <v>"ml" STD_RIGHT_ARROW</v>
       </c>
@@ -2888,15 +2944,15 @@
         <f t="shared" si="2"/>
         <v>/* NNNN */  UNIT_CONV(constFactorMlQtus,          divide,      "ml" STD_RIGHT_ARROW "qt" STD_US,                            "ml" STD_RIGHT_ARROW                                        ),</v>
       </c>
-      <c r="I19" s="53">
+      <c r="I19" s="52">
         <f>VLOOKUP(A19,Factors!D:G,4,0)</f>
         <v>946.35294599999997</v>
       </c>
-      <c r="J19" s="53" t="str">
+      <c r="J19" s="52" t="str">
         <f t="shared" si="3"/>
         <v>9.463529460000000000000000000000000000000000000000000000e+02</v>
       </c>
-      <c r="K19" s="56" t="str">
+      <c r="K19" s="55" t="str">
         <f>VLOOKUP(A19,Factors!D:N,11,0)</f>
         <v>QtusMl</v>
       </c>
@@ -2916,22 +2972,22 @@
       <c r="B20" s="43" t="s">
         <v>21</v>
       </c>
-      <c r="C20" s="91" t="s">
+      <c r="C20" s="90" t="s">
         <v>70</v>
       </c>
       <c r="D20" s="40" t="str">
         <f>VLOOKUP(A20,Factors!D:K,8,0)</f>
         <v>constFactorMlTbspc</v>
       </c>
-      <c r="E20" s="53" t="str">
+      <c r="E20" s="52" t="str">
         <f>VLOOKUP(A20,Factors!D:N,10,0)</f>
         <v xml:space="preserve">  divide</v>
       </c>
-      <c r="F20" s="55" t="str">
+      <c r="F20" s="54" t="str">
         <f t="shared" si="0"/>
         <v>"ml" STD_RIGHT_ARROW "Tbsp" STD_US STD_SUB_c</v>
       </c>
-      <c r="G20" s="55" t="str">
+      <c r="G20" s="54" t="str">
         <f t="shared" si="1"/>
         <v>"ml" STD_RIGHT_ARROW</v>
       </c>
@@ -2939,15 +2995,15 @@
         <f t="shared" si="2"/>
         <v>/* NNNN */  UNIT_CONV(constFactorMlTbspc,         divide,      "ml" STD_RIGHT_ARROW "Tbsp" STD_US STD_SUB_c,                "ml" STD_RIGHT_ARROW                                        ),</v>
       </c>
-      <c r="I20" s="53">
+      <c r="I20" s="52">
         <f>VLOOKUP(A20,Factors!D:G,4,0)</f>
         <v>14.78676478125</v>
       </c>
-      <c r="J20" s="53" t="str">
+      <c r="J20" s="52" t="str">
         <f t="shared" si="3"/>
         <v>1.478676478125000000000000000000000000000000000000000000e+01</v>
       </c>
-      <c r="K20" s="56" t="str">
+      <c r="K20" s="55" t="str">
         <f>VLOOKUP(A20,Factors!D:N,11,0)</f>
         <v>TbspcMl</v>
       </c>
@@ -2967,22 +3023,22 @@
       <c r="B21" s="43" t="s">
         <v>49</v>
       </c>
-      <c r="C21" s="91" t="s">
+      <c r="C21" s="90" t="s">
         <v>70</v>
       </c>
       <c r="D21" s="40" t="str">
         <f>VLOOKUP(A21,Factors!D:K,8,0)</f>
         <v>constFactorMlTbspuk</v>
       </c>
-      <c r="E21" s="53" t="str">
+      <c r="E21" s="52" t="str">
         <f>VLOOKUP(A21,Factors!D:N,10,0)</f>
         <v xml:space="preserve">  divide</v>
       </c>
-      <c r="F21" s="55" t="str">
+      <c r="F21" s="54" t="str">
         <f t="shared" si="0"/>
         <v>"ml" STD_RIGHT_ARROW "Tbsp" STD_UK</v>
       </c>
-      <c r="G21" s="55" t="str">
+      <c r="G21" s="54" t="str">
         <f t="shared" si="1"/>
         <v>"ml" STD_RIGHT_ARROW</v>
       </c>
@@ -2990,15 +3046,15 @@
         <f t="shared" si="2"/>
         <v>/* NNNN */  UNIT_CONV(constFactorMlTbspuk,        divide,      "ml" STD_RIGHT_ARROW "Tbsp" STD_UK,                          "ml" STD_RIGHT_ARROW                                        ),</v>
       </c>
-      <c r="I21" s="53">
+      <c r="I21" s="52">
         <f>VLOOKUP(A21,Factors!D:G,4,0)</f>
         <v>17.758164062500001</v>
       </c>
-      <c r="J21" s="53" t="str">
+      <c r="J21" s="52" t="str">
         <f t="shared" si="3"/>
         <v>1.775816406250000000000000000000000000000000000000000000e+01</v>
       </c>
-      <c r="K21" s="56" t="str">
+      <c r="K21" s="55" t="str">
         <f>VLOOKUP(A21,Factors!D:N,11,0)</f>
         <v>TbspukMl</v>
       </c>
@@ -3018,22 +3074,22 @@
       <c r="B22" s="43" t="s">
         <v>25</v>
       </c>
-      <c r="C22" s="91" t="s">
+      <c r="C22" s="90" t="s">
         <v>70</v>
       </c>
       <c r="D22" s="40" t="str">
         <f>VLOOKUP(A22,Factors!D:K,8,0)</f>
         <v>constFactorMlTspc</v>
       </c>
-      <c r="E22" s="53" t="str">
+      <c r="E22" s="52" t="str">
         <f>VLOOKUP(A22,Factors!D:N,10,0)</f>
         <v xml:space="preserve">  divide</v>
       </c>
-      <c r="F22" s="55" t="str">
+      <c r="F22" s="54" t="str">
         <f t="shared" si="0"/>
         <v>"ml" STD_RIGHT_ARROW "tsp" STD_US STD_SUB_c</v>
       </c>
-      <c r="G22" s="55" t="str">
+      <c r="G22" s="54" t="str">
         <f t="shared" si="1"/>
         <v>"ml" STD_RIGHT_ARROW</v>
       </c>
@@ -3041,15 +3097,15 @@
         <f t="shared" si="2"/>
         <v>/* NNNN */  UNIT_CONV(constFactorMlTspc,          divide,      "ml" STD_RIGHT_ARROW "tsp" STD_US STD_SUB_c,                 "ml" STD_RIGHT_ARROW                                        ),</v>
       </c>
-      <c r="I22" s="53">
+      <c r="I22" s="52">
         <f>VLOOKUP(A22,Factors!D:G,4,0)</f>
         <v>4.9289215937500002</v>
       </c>
-      <c r="J22" s="53" t="str">
+      <c r="J22" s="52" t="str">
         <f t="shared" si="3"/>
         <v>4.928921593750000000000000000000000000000000000000000000e+00</v>
       </c>
-      <c r="K22" s="56" t="str">
+      <c r="K22" s="55" t="str">
         <f>VLOOKUP(A22,Factors!D:N,11,0)</f>
         <v>TspcMl</v>
       </c>
@@ -3069,22 +3125,22 @@
       <c r="B23" s="43" t="s">
         <v>53</v>
       </c>
-      <c r="C23" s="91" t="s">
+      <c r="C23" s="90" t="s">
         <v>70</v>
       </c>
       <c r="D23" s="40" t="str">
         <f>VLOOKUP(A23,Factors!D:K,8,0)</f>
         <v>constFactorMlTspuk</v>
       </c>
-      <c r="E23" s="53" t="str">
+      <c r="E23" s="52" t="str">
         <f>VLOOKUP(A23,Factors!D:N,10,0)</f>
         <v xml:space="preserve">  divide</v>
       </c>
-      <c r="F23" s="55" t="str">
+      <c r="F23" s="54" t="str">
         <f t="shared" si="0"/>
         <v>"ml" STD_RIGHT_ARROW "tsp" STD_UK</v>
       </c>
-      <c r="G23" s="55" t="str">
+      <c r="G23" s="54" t="str">
         <f t="shared" si="1"/>
         <v>"ml" STD_RIGHT_ARROW</v>
       </c>
@@ -3092,15 +3148,15 @@
         <f t="shared" si="2"/>
         <v>/* NNNN */  UNIT_CONV(constFactorMlTspuk,         divide,      "ml" STD_RIGHT_ARROW "tsp" STD_UK,                           "ml" STD_RIGHT_ARROW                                        ),</v>
       </c>
-      <c r="I23" s="53">
+      <c r="I23" s="52">
         <f>VLOOKUP(A23,Factors!D:G,4,0)</f>
         <v>5.9193880208333338</v>
       </c>
-      <c r="J23" s="53" t="str">
+      <c r="J23" s="52" t="str">
         <f t="shared" si="3"/>
         <v>5.919388020833330000000000000000000000000000000000000000e+00</v>
       </c>
-      <c r="K23" s="56" t="str">
+      <c r="K23" s="55" t="str">
         <f>VLOOKUP(A23,Factors!D:N,11,0)</f>
         <v>TspukMl</v>
       </c>
@@ -3120,22 +3176,22 @@
       <c r="B24" s="43" t="s">
         <v>1</v>
       </c>
-      <c r="C24" s="91" t="s">
+      <c r="C24" s="90" t="s">
         <v>70</v>
       </c>
       <c r="D24" s="40" t="str">
         <f>VLOOKUP(A24,Factors!D:K,8,0)</f>
         <v>constFactorPintlqMl</v>
       </c>
-      <c r="E24" s="53" t="str">
+      <c r="E24" s="52" t="str">
         <f>VLOOKUP(A24,Factors!D:N,10,0)</f>
         <v>multiply</v>
       </c>
-      <c r="F24" s="55" t="str">
+      <c r="F24" s="54" t="str">
         <f t="shared" si="0"/>
         <v>"pint" STD_SUB_l STD_SUB_i STD_SUB_q STD_RIGHT_ARROW "ml"</v>
       </c>
-      <c r="G24" s="55" t="str">
+      <c r="G24" s="54" t="str">
         <f t="shared" si="1"/>
         <v>"pint" STD_SUB_l STD_SUB_i STD_SUB_q STD_RIGHT_ARROW</v>
       </c>
@@ -3143,15 +3199,15 @@
         <f t="shared" si="2"/>
         <v>/* NNNN */  UNIT_CONV(constFactorPintlqMl,      multiply,      "pint" STD_SUB_l STD_SUB_i STD_SUB_q STD_RIGHT_ARROW "ml",   "pint" STD_SUB_l STD_SUB_i STD_SUB_q STD_RIGHT_ARROW        ),</v>
       </c>
-      <c r="I24" s="53">
+      <c r="I24" s="52">
         <f>VLOOKUP(A24,Factors!D:G,4,0)</f>
         <v>473.17647299999999</v>
       </c>
-      <c r="J24" s="53" t="str">
+      <c r="J24" s="52" t="str">
         <f t="shared" si="3"/>
         <v>4.731764730000000000000000000000000000000000000000000000e+02</v>
       </c>
-      <c r="K24" s="56" t="str">
+      <c r="K24" s="55" t="str">
         <f>VLOOKUP(A24,Factors!D:N,11,0)</f>
         <v>PintlqMl</v>
       </c>
@@ -3171,22 +3227,22 @@
       <c r="B25" s="43" t="s">
         <v>29</v>
       </c>
-      <c r="C25" s="91" t="s">
+      <c r="C25" s="90" t="s">
         <v>70</v>
       </c>
       <c r="D25" s="40" t="str">
         <f>VLOOKUP(A25,Factors!D:K,8,0)</f>
         <v>constFactorPintukMl</v>
       </c>
-      <c r="E25" s="53" t="str">
+      <c r="E25" s="52" t="str">
         <f>VLOOKUP(A25,Factors!D:N,10,0)</f>
         <v>multiply</v>
       </c>
-      <c r="F25" s="55" t="str">
+      <c r="F25" s="54" t="str">
         <f t="shared" si="0"/>
         <v>"pint" STD_UK STD_RIGHT_ARROW "ml"</v>
       </c>
-      <c r="G25" s="55" t="str">
+      <c r="G25" s="54" t="str">
         <f t="shared" si="1"/>
         <v>"pint" STD_UK STD_RIGHT_ARROW</v>
       </c>
@@ -3194,15 +3250,15 @@
         <f t="shared" si="2"/>
         <v>/* NNNN */  UNIT_CONV(constFactorPintukMl,      multiply,      "pint" STD_UK STD_RIGHT_ARROW "ml",                          "pint" STD_UK STD_RIGHT_ARROW                               ),</v>
       </c>
-      <c r="I25" s="53">
+      <c r="I25" s="52">
         <f>VLOOKUP(A25,Factors!D:G,4,0)</f>
         <v>568.26125000000002</v>
       </c>
-      <c r="J25" s="53" t="str">
+      <c r="J25" s="52" t="str">
         <f t="shared" si="3"/>
         <v>5.682612500000000000000000000000000000000000000000000000e+02</v>
       </c>
-      <c r="K25" s="56" t="str">
+      <c r="K25" s="55" t="str">
         <f>VLOOKUP(A25,Factors!D:N,11,0)</f>
         <v>PintukMl</v>
       </c>
@@ -3222,22 +3278,22 @@
       <c r="B26" s="43" t="s">
         <v>33</v>
       </c>
-      <c r="C26" s="91" t="s">
+      <c r="C26" s="90" t="s">
         <v>70</v>
       </c>
       <c r="D26" s="40" t="str">
         <f>VLOOKUP(A26,Factors!D:K,8,0)</f>
         <v>constFactorQtMl</v>
       </c>
-      <c r="E26" s="53" t="str">
+      <c r="E26" s="52" t="str">
         <f>VLOOKUP(A26,Factors!D:N,10,0)</f>
         <v>multiply</v>
       </c>
-      <c r="F26" s="55" t="str">
+      <c r="F26" s="54" t="str">
         <f t="shared" si="0"/>
         <v>"qt" STD_UK STD_RIGHT_ARROW "ml"</v>
       </c>
-      <c r="G26" s="55" t="str">
+      <c r="G26" s="54" t="str">
         <f t="shared" si="1"/>
         <v>"qt" STD_UK STD_RIGHT_ARROW</v>
       </c>
@@ -3245,15 +3301,15 @@
         <f t="shared" si="2"/>
         <v>/* NNNN */  UNIT_CONV(constFactorQtMl,          multiply,      "qt" STD_UK STD_RIGHT_ARROW "ml",                            "qt" STD_UK STD_RIGHT_ARROW                                 ),</v>
       </c>
-      <c r="I26" s="53">
+      <c r="I26" s="52">
         <f>VLOOKUP(A26,Factors!D:G,4,0)</f>
         <v>1136.5225</v>
       </c>
-      <c r="J26" s="53" t="str">
+      <c r="J26" s="52" t="str">
         <f t="shared" si="3"/>
         <v>1.136522500000000000000000000000000000000000000000000000e+03</v>
       </c>
-      <c r="K26" s="56" t="str">
+      <c r="K26" s="55" t="str">
         <f>VLOOKUP(A26,Factors!D:N,11,0)</f>
         <v>QtMl</v>
       </c>
@@ -3273,22 +3329,22 @@
       <c r="B27" s="43" t="s">
         <v>5</v>
       </c>
-      <c r="C27" s="91" t="s">
+      <c r="C27" s="90" t="s">
         <v>70</v>
       </c>
       <c r="D27" s="40" t="str">
         <f>VLOOKUP(A27,Factors!D:K,8,0)</f>
         <v>constFactorQtusMl</v>
       </c>
-      <c r="E27" s="53" t="str">
+      <c r="E27" s="52" t="str">
         <f>VLOOKUP(A27,Factors!D:N,10,0)</f>
         <v>multiply</v>
       </c>
-      <c r="F27" s="55" t="str">
+      <c r="F27" s="54" t="str">
         <f t="shared" si="0"/>
         <v>"qt" STD_US STD_RIGHT_ARROW "ml"</v>
       </c>
-      <c r="G27" s="55" t="str">
+      <c r="G27" s="54" t="str">
         <f t="shared" si="1"/>
         <v>"qt" STD_US STD_RIGHT_ARROW</v>
       </c>
@@ -3296,15 +3352,15 @@
         <f t="shared" si="2"/>
         <v>/* NNNN */  UNIT_CONV(constFactorQtusMl,        multiply,      "qt" STD_US STD_RIGHT_ARROW "ml",                            "qt" STD_US STD_RIGHT_ARROW                                 ),</v>
       </c>
-      <c r="I27" s="53">
+      <c r="I27" s="52">
         <f>VLOOKUP(A27,Factors!D:G,4,0)</f>
         <v>946.35294599999997</v>
       </c>
-      <c r="J27" s="53" t="str">
+      <c r="J27" s="52" t="str">
         <f t="shared" si="3"/>
         <v>9.463529460000000000000000000000000000000000000000000000e+02</v>
       </c>
-      <c r="K27" s="56" t="str">
+      <c r="K27" s="55" t="str">
         <f>VLOOKUP(A27,Factors!D:N,11,0)</f>
         <v>QtusMl</v>
       </c>
@@ -3324,22 +3380,22 @@
       <c r="B28" s="43" t="s">
         <v>15</v>
       </c>
-      <c r="C28" s="91" t="s">
+      <c r="C28" s="90" t="s">
         <v>70</v>
       </c>
       <c r="D28" s="40" t="str">
         <f>VLOOKUP(A28,Factors!D:K,8,0)</f>
         <v>constFactorTbspcFzus</v>
       </c>
-      <c r="E28" s="53" t="str">
+      <c r="E28" s="52" t="str">
         <f>VLOOKUP(A28,Factors!D:N,10,0)</f>
         <v xml:space="preserve">  divide</v>
       </c>
-      <c r="F28" s="55" t="str">
+      <c r="F28" s="54" t="str">
         <f t="shared" si="0"/>
         <v>"Tbsp" STD_US STD_SUB_c STD_RIGHT_ARROW "floz" STD_US</v>
       </c>
-      <c r="G28" s="55" t="str">
+      <c r="G28" s="54" t="str">
         <f t="shared" si="1"/>
         <v>"Tbsp" STD_US STD_SUB_c STD_RIGHT_ARROW</v>
       </c>
@@ -3347,15 +3403,15 @@
         <f t="shared" si="2"/>
         <v>/* NNNN */  UNIT_CONV(constFactorTbspcFzus,       divide,      "Tbsp" STD_US STD_SUB_c STD_RIGHT_ARROW "floz" STD_US,       "Tbsp" STD_US STD_SUB_c STD_RIGHT_ARROW                     ),</v>
       </c>
-      <c r="I28" s="53">
+      <c r="I28" s="52">
         <f>VLOOKUP(A28,Factors!D:G,4,0)</f>
         <v>2</v>
       </c>
-      <c r="J28" s="53" t="str">
+      <c r="J28" s="52" t="str">
         <f t="shared" si="3"/>
         <v>2.000000000000000000000000000000000000000000000000000000e+00</v>
       </c>
-      <c r="K28" s="56" t="str">
+      <c r="K28" s="55" t="str">
         <f>VLOOKUP(A28,Factors!D:N,11,0)</f>
         <v>FzusTbspc</v>
       </c>
@@ -3375,22 +3431,22 @@
       <c r="B29" s="43" t="s">
         <v>23</v>
       </c>
-      <c r="C29" s="91" t="s">
+      <c r="C29" s="90" t="s">
         <v>70</v>
       </c>
       <c r="D29" s="40" t="str">
         <f>VLOOKUP(A29,Factors!D:K,8,0)</f>
         <v>constFactorTbspcMl</v>
       </c>
-      <c r="E29" s="53" t="str">
+      <c r="E29" s="52" t="str">
         <f>VLOOKUP(A29,Factors!D:N,10,0)</f>
         <v>multiply</v>
       </c>
-      <c r="F29" s="55" t="str">
+      <c r="F29" s="54" t="str">
         <f t="shared" si="0"/>
         <v>"Tbsp" STD_US STD_SUB_c STD_RIGHT_ARROW "ml"</v>
       </c>
-      <c r="G29" s="55" t="str">
+      <c r="G29" s="54" t="str">
         <f t="shared" si="1"/>
         <v>"Tbsp" STD_US STD_SUB_c STD_RIGHT_ARROW</v>
       </c>
@@ -3398,15 +3454,15 @@
         <f t="shared" si="2"/>
         <v>/* NNNN */  UNIT_CONV(constFactorTbspcMl,       multiply,      "Tbsp" STD_US STD_SUB_c STD_RIGHT_ARROW "ml",                "Tbsp" STD_US STD_SUB_c STD_RIGHT_ARROW                     ),</v>
       </c>
-      <c r="I29" s="53">
+      <c r="I29" s="52">
         <f>VLOOKUP(A29,Factors!D:G,4,0)</f>
         <v>14.78676478125</v>
       </c>
-      <c r="J29" s="53" t="str">
+      <c r="J29" s="52" t="str">
         <f t="shared" si="3"/>
         <v>1.478676478125000000000000000000000000000000000000000000e+01</v>
       </c>
-      <c r="K29" s="56" t="str">
+      <c r="K29" s="55" t="str">
         <f>VLOOKUP(A29,Factors!D:N,11,0)</f>
         <v>TbspcMl</v>
       </c>
@@ -3426,22 +3482,22 @@
       <c r="B30" s="43" t="s">
         <v>43</v>
       </c>
-      <c r="C30" s="91" t="s">
+      <c r="C30" s="90" t="s">
         <v>70</v>
       </c>
       <c r="D30" s="40" t="str">
         <f>VLOOKUP(A30,Factors!D:K,8,0)</f>
         <v>constFactorTbspukFzuk</v>
       </c>
-      <c r="E30" s="53" t="str">
+      <c r="E30" s="52" t="str">
         <f>VLOOKUP(A30,Factors!D:N,10,0)</f>
         <v xml:space="preserve">  divide</v>
       </c>
-      <c r="F30" s="55" t="str">
+      <c r="F30" s="54" t="str">
         <f t="shared" si="0"/>
         <v>"Tbsp" STD_UK STD_RIGHT_ARROW "floz" STD_UK</v>
       </c>
-      <c r="G30" s="55" t="str">
+      <c r="G30" s="54" t="str">
         <f t="shared" si="1"/>
         <v>"Tbsp" STD_UK STD_RIGHT_ARROW</v>
       </c>
@@ -3449,15 +3505,15 @@
         <f t="shared" si="2"/>
         <v>/* NNNN */  UNIT_CONV(constFactorTbspukFzuk,      divide,      "Tbsp" STD_UK STD_RIGHT_ARROW "floz" STD_UK,                 "Tbsp" STD_UK STD_RIGHT_ARROW                               ),</v>
       </c>
-      <c r="I30" s="53">
+      <c r="I30" s="52">
         <f>VLOOKUP(A30,Factors!D:G,4,0)</f>
         <v>1.6</v>
       </c>
-      <c r="J30" s="53" t="str">
+      <c r="J30" s="52" t="str">
         <f t="shared" si="3"/>
         <v>1.600000000000000000000000000000000000000000000000000000e+00</v>
       </c>
-      <c r="K30" s="56" t="str">
+      <c r="K30" s="55" t="str">
         <f>VLOOKUP(A30,Factors!D:N,11,0)</f>
         <v>FzukTbspuk</v>
       </c>
@@ -3477,22 +3533,22 @@
       <c r="B31" s="43" t="s">
         <v>51</v>
       </c>
-      <c r="C31" s="91" t="s">
+      <c r="C31" s="90" t="s">
         <v>70</v>
       </c>
       <c r="D31" s="40" t="str">
         <f>VLOOKUP(A31,Factors!D:K,8,0)</f>
         <v>constFactorTbspukMl</v>
       </c>
-      <c r="E31" s="53" t="str">
+      <c r="E31" s="52" t="str">
         <f>VLOOKUP(A31,Factors!D:N,10,0)</f>
         <v>multiply</v>
       </c>
-      <c r="F31" s="55" t="str">
+      <c r="F31" s="54" t="str">
         <f t="shared" si="0"/>
         <v>"Tbsp" STD_UK STD_RIGHT_ARROW "ml"</v>
       </c>
-      <c r="G31" s="55" t="str">
+      <c r="G31" s="54" t="str">
         <f t="shared" si="1"/>
         <v>"Tbsp" STD_UK STD_RIGHT_ARROW</v>
       </c>
@@ -3500,15 +3556,15 @@
         <f t="shared" si="2"/>
         <v>/* NNNN */  UNIT_CONV(constFactorTbspukMl,      multiply,      "Tbsp" STD_UK STD_RIGHT_ARROW "ml",                          "Tbsp" STD_UK STD_RIGHT_ARROW                               ),</v>
       </c>
-      <c r="I31" s="53">
+      <c r="I31" s="52">
         <f>VLOOKUP(A31,Factors!D:G,4,0)</f>
         <v>17.758164062500001</v>
       </c>
-      <c r="J31" s="53" t="str">
+      <c r="J31" s="52" t="str">
         <f t="shared" si="3"/>
         <v>1.775816406250000000000000000000000000000000000000000000e+01</v>
       </c>
-      <c r="K31" s="56" t="str">
+      <c r="K31" s="55" t="str">
         <f>VLOOKUP(A31,Factors!D:N,11,0)</f>
         <v>TbspukMl</v>
       </c>
@@ -3528,22 +3584,22 @@
       <c r="B32" s="43" t="s">
         <v>59</v>
       </c>
-      <c r="C32" s="91" t="s">
+      <c r="C32" s="90" t="s">
         <v>70</v>
       </c>
       <c r="D32" s="40" t="str">
         <f>VLOOKUP(A32,Factors!D:K,8,0)</f>
         <v>constFactorTspcFzus</v>
       </c>
-      <c r="E32" s="53" t="str">
+      <c r="E32" s="52" t="str">
         <f>VLOOKUP(A32,Factors!D:N,10,0)</f>
         <v xml:space="preserve">  divide</v>
       </c>
-      <c r="F32" s="55" t="str">
+      <c r="F32" s="54" t="str">
         <f t="shared" si="0"/>
         <v>"tsp" STD_US STD_SUB_c STD_RIGHT_ARROW "floz" STD_US</v>
       </c>
-      <c r="G32" s="55" t="str">
+      <c r="G32" s="54" t="str">
         <f t="shared" si="1"/>
         <v>"tsp" STD_US STD_SUB_c STD_RIGHT_ARROW</v>
       </c>
@@ -3551,15 +3607,15 @@
         <f t="shared" si="2"/>
         <v>/* NNNN */  UNIT_CONV(constFactorTspcFzus,        divide,      "tsp" STD_US STD_SUB_c STD_RIGHT_ARROW "floz" STD_US,        "tsp" STD_US STD_SUB_c STD_RIGHT_ARROW                      ),</v>
       </c>
-      <c r="I32" s="53">
+      <c r="I32" s="52">
         <f>VLOOKUP(A32,Factors!D:G,4,0)</f>
         <v>6</v>
       </c>
-      <c r="J32" s="53" t="str">
+      <c r="J32" s="52" t="str">
         <f t="shared" si="3"/>
         <v>6.000000000000000000000000000000000000000000000000000000e+00</v>
       </c>
-      <c r="K32" s="56" t="str">
+      <c r="K32" s="55" t="str">
         <f>VLOOKUP(A32,Factors!D:N,11,0)</f>
         <v>FzusTspc</v>
       </c>
@@ -3579,22 +3635,22 @@
       <c r="B33" s="43" t="s">
         <v>27</v>
       </c>
-      <c r="C33" s="91" t="s">
+      <c r="C33" s="90" t="s">
         <v>70</v>
       </c>
       <c r="D33" s="40" t="str">
         <f>VLOOKUP(A33,Factors!D:K,8,0)</f>
         <v>constFactorTspcMl</v>
       </c>
-      <c r="E33" s="53" t="str">
+      <c r="E33" s="52" t="str">
         <f>VLOOKUP(A33,Factors!D:N,10,0)</f>
         <v>multiply</v>
       </c>
-      <c r="F33" s="55" t="str">
+      <c r="F33" s="54" t="str">
         <f t="shared" si="0"/>
         <v>"tsp" STD_US STD_SUB_c STD_RIGHT_ARROW "ml"</v>
       </c>
-      <c r="G33" s="55" t="str">
+      <c r="G33" s="54" t="str">
         <f t="shared" si="1"/>
         <v>"tsp" STD_US STD_SUB_c STD_RIGHT_ARROW</v>
       </c>
@@ -3602,15 +3658,15 @@
         <f t="shared" si="2"/>
         <v>/* NNNN */  UNIT_CONV(constFactorTspcMl,        multiply,      "tsp" STD_US STD_SUB_c STD_RIGHT_ARROW "ml",                 "tsp" STD_US STD_SUB_c STD_RIGHT_ARROW                      ),</v>
       </c>
-      <c r="I33" s="53">
+      <c r="I33" s="52">
         <f>VLOOKUP(A33,Factors!D:G,4,0)</f>
         <v>4.9289215937500002</v>
       </c>
-      <c r="J33" s="53" t="str">
+      <c r="J33" s="52" t="str">
         <f t="shared" si="3"/>
         <v>4.928921593750000000000000000000000000000000000000000000e+00</v>
       </c>
-      <c r="K33" s="56" t="str">
+      <c r="K33" s="55" t="str">
         <f>VLOOKUP(A33,Factors!D:N,11,0)</f>
         <v>TspcMl</v>
       </c>
@@ -3630,22 +3686,22 @@
       <c r="B34" s="43" t="s">
         <v>61</v>
       </c>
-      <c r="C34" s="91" t="s">
+      <c r="C34" s="90" t="s">
         <v>70</v>
       </c>
       <c r="D34" s="40" t="str">
         <f>VLOOKUP(A34,Factors!D:K,8,0)</f>
         <v>constFactorTspukFzuk</v>
       </c>
-      <c r="E34" s="53" t="str">
+      <c r="E34" s="52" t="str">
         <f>VLOOKUP(A34,Factors!D:N,10,0)</f>
         <v xml:space="preserve">  divide</v>
       </c>
-      <c r="F34" s="55" t="str">
+      <c r="F34" s="54" t="str">
         <f t="shared" si="0"/>
         <v>"tsp" STD_UK STD_RIGHT_ARROW "floz" STD_UK</v>
       </c>
-      <c r="G34" s="55" t="str">
+      <c r="G34" s="54" t="str">
         <f t="shared" si="1"/>
         <v>"tsp" STD_UK STD_RIGHT_ARROW</v>
       </c>
@@ -3653,15 +3709,15 @@
         <f t="shared" si="2"/>
         <v>/* NNNN */  UNIT_CONV(constFactorTspukFzuk,       divide,      "tsp" STD_UK STD_RIGHT_ARROW "floz" STD_UK,                  "tsp" STD_UK STD_RIGHT_ARROW                                ),</v>
       </c>
-      <c r="I34" s="53">
+      <c r="I34" s="52">
         <f>VLOOKUP(A34,Factors!D:G,4,0)</f>
         <v>4.8</v>
       </c>
-      <c r="J34" s="53" t="str">
+      <c r="J34" s="52" t="str">
         <f t="shared" si="3"/>
         <v>4.800000000000000000000000000000000000000000000000000000e+00</v>
       </c>
-      <c r="K34" s="56" t="str">
+      <c r="K34" s="55" t="str">
         <f>VLOOKUP(A34,Factors!D:N,11,0)</f>
         <v>FzukTspuk</v>
       </c>
@@ -3681,47 +3737,47 @@
       <c r="B35" s="43" t="s">
         <v>55</v>
       </c>
-      <c r="C35" s="91" t="s">
+      <c r="C35" s="90" t="s">
         <v>70</v>
       </c>
       <c r="D35" s="40" t="str">
         <f>VLOOKUP(A35,Factors!D:K,8,0)</f>
         <v>constFactorTspukMl</v>
       </c>
-      <c r="E35" s="53" t="str">
+      <c r="E35" s="52" t="str">
         <f>VLOOKUP(A35,Factors!D:N,10,0)</f>
         <v>multiply</v>
       </c>
-      <c r="F35" s="55" t="str">
-        <f t="shared" ref="F35:F42" si="6" xml:space="preserve"> VLOOKUP(A35,stdform,2,0)</f>
+      <c r="F35" s="54" t="str">
+        <f t="shared" ref="F35:F46" si="6" xml:space="preserve"> VLOOKUP(A35,stdform,2,0)</f>
         <v>"tsp" STD_UK STD_RIGHT_ARROW "ml"</v>
       </c>
-      <c r="G35" s="55" t="str">
-        <f t="shared" ref="G35:G42" si="7">MID(F35,1,SEARCH("STD_RIGHT_ARROW",F35)-2)&amp;" STD_RIGHT_ARROW"</f>
+      <c r="G35" s="54" t="str">
+        <f t="shared" ref="G35:G46" si="7">MID(F35,1,SEARCH("STD_RIGHT_ARROW",F35)-2)&amp;" STD_RIGHT_ARROW"</f>
         <v>"tsp" STD_UK STD_RIGHT_ARROW</v>
       </c>
       <c r="H35" s="30" t="str">
-        <f t="shared" ref="H35:H42" si="8">"/* NNNN */  UNIT_CONV("&amp;D35&amp;","&amp;REPT(CHAR(32),21-LEN(D35))&amp;"    "&amp;E35&amp;",      "&amp;F35&amp;","&amp;REPT(CHAR(32),60-LEN(F35))&amp;G35&amp;REPT(CHAR(32),60-LEN(G35))&amp;"),"</f>
+        <f t="shared" ref="H35:H46" si="8">"/* NNNN */  UNIT_CONV("&amp;D35&amp;","&amp;REPT(CHAR(32),21-LEN(D35))&amp;"    "&amp;E35&amp;",      "&amp;F35&amp;","&amp;REPT(CHAR(32),60-LEN(F35))&amp;G35&amp;REPT(CHAR(32),60-LEN(G35))&amp;"),"</f>
         <v>/* NNNN */  UNIT_CONV(constFactorTspukMl,       multiply,      "tsp" STD_UK STD_RIGHT_ARROW "ml",                           "tsp" STD_UK STD_RIGHT_ARROW                                ),</v>
       </c>
-      <c r="I35" s="53">
+      <c r="I35" s="52">
         <f>VLOOKUP(A35,Factors!D:G,4,0)</f>
         <v>5.9193880208333338</v>
       </c>
-      <c r="J35" s="53" t="str">
-        <f t="shared" ref="J35:J42" si="9">SUBSTITUTE(TEXT(I35,"0.000000000000000000000000000000000000000000000000000000E+00"),"E","e")</f>
+      <c r="J35" s="52" t="str">
+        <f t="shared" ref="J35:J46" si="9">SUBSTITUTE(TEXT(I35,"0.000000000000000000000000000000000000000000000000000000E+00"),"E","e")</f>
         <v>5.919388020833330000000000000000000000000000000000000000e+00</v>
       </c>
-      <c r="K35" s="56" t="str">
+      <c r="K35" s="55" t="str">
         <f>VLOOKUP(A35,Factors!D:N,11,0)</f>
         <v>TspukMl</v>
       </c>
       <c r="L35" s="31" t="str">
-        <f t="shared" ref="L35:L42" si="10">IF(E35="multiply","  generateConstantArray("&amp;CHAR(34)&amp;K35&amp;CHAR(34)&amp;","&amp;REPT(CHAR(32),14-LEN(K35))&amp;CHAR(34)&amp;"+"&amp;J35&amp;CHAR(34)&amp;");","")</f>
+        <f t="shared" ref="L35:L46" si="10">IF(E35="multiply","  generateConstantArray("&amp;CHAR(34)&amp;K35&amp;CHAR(34)&amp;","&amp;REPT(CHAR(32),14-LEN(K35))&amp;CHAR(34)&amp;"+"&amp;J35&amp;CHAR(34)&amp;");","")</f>
         <v xml:space="preserve">  generateConstantArray("TspukMl",       "+5.919388020833330000000000000000000000000000000000000000e+00");</v>
       </c>
       <c r="N35" s="41" t="str">
-        <f t="shared" ref="N35:N42" si="11">"    ["&amp;D35&amp;"] = "&amp;CHAR(38)&amp;"const_"&amp;K35&amp;","</f>
+        <f t="shared" ref="N35:N46" si="11">"    ["&amp;D35&amp;"] = "&amp;CHAR(38)&amp;"const_"&amp;K35&amp;","</f>
         <v xml:space="preserve">    [constFactorTspukMl] = &amp;const_TspukMl,</v>
       </c>
     </row>
@@ -3732,22 +3788,22 @@
       <c r="B36" s="44" t="s">
         <v>193</v>
       </c>
-      <c r="C36" s="92" t="s">
+      <c r="C36" s="91" t="s">
         <v>70</v>
       </c>
       <c r="D36" s="40" t="str">
         <f>VLOOKUP(A36,Factors!D:K,8,0)</f>
         <v>constFactorMlIn3</v>
       </c>
-      <c r="E36" s="53" t="str">
+      <c r="E36" s="52" t="str">
         <f>VLOOKUP(A36,Factors!D:N,10,0)</f>
         <v xml:space="preserve">  divide</v>
       </c>
-      <c r="F36" s="55" t="str">
+      <c r="F36" s="54" t="str">
         <f t="shared" si="6"/>
         <v>"m" STD_litre STD_RIGHT_ARROW "in" STD_SUP_3</v>
       </c>
-      <c r="G36" s="55" t="str">
+      <c r="G36" s="54" t="str">
         <f t="shared" si="7"/>
         <v>"m" STD_litre STD_RIGHT_ARROW</v>
       </c>
@@ -3755,15 +3811,15 @@
         <f t="shared" si="8"/>
         <v>/* NNNN */  UNIT_CONV(constFactorMlIn3,           divide,      "m" STD_litre STD_RIGHT_ARROW "in" STD_SUP_3,                "m" STD_litre STD_RIGHT_ARROW                               ),</v>
       </c>
-      <c r="I36" s="53">
+      <c r="I36" s="52">
         <f>VLOOKUP(A36,Factors!D:G,4,0)</f>
         <v>16.387063999999999</v>
       </c>
-      <c r="J36" s="53" t="str">
+      <c r="J36" s="52" t="str">
         <f t="shared" si="9"/>
         <v>1.638706400000000000000000000000000000000000000000000000e+01</v>
       </c>
-      <c r="K36" s="56" t="str">
+      <c r="K36" s="55" t="str">
         <f>VLOOKUP(A36,Factors!D:N,11,0)</f>
         <v>In3Ml</v>
       </c>
@@ -3783,22 +3839,22 @@
       <c r="B37" s="44" t="s">
         <v>194</v>
       </c>
-      <c r="C37" s="92" t="s">
+      <c r="C37" s="91" t="s">
         <v>70</v>
       </c>
       <c r="D37" s="40" t="str">
         <f>VLOOKUP(A37,Factors!D:K,8,0)</f>
         <v>constFactorIn3Ml</v>
       </c>
-      <c r="E37" s="53" t="str">
+      <c r="E37" s="52" t="str">
         <f>VLOOKUP(A37,Factors!D:N,10,0)</f>
         <v>multiply</v>
       </c>
-      <c r="F37" s="55" t="str">
+      <c r="F37" s="54" t="str">
         <f t="shared" si="6"/>
         <v>"in" STD_SUP_3 STD_RIGHT_ARROW "m" STD_litre</v>
       </c>
-      <c r="G37" s="55" t="str">
+      <c r="G37" s="54" t="str">
         <f t="shared" si="7"/>
         <v>"in" STD_SUP_3 STD_RIGHT_ARROW</v>
       </c>
@@ -3806,15 +3862,15 @@
         <f t="shared" si="8"/>
         <v>/* NNNN */  UNIT_CONV(constFactorIn3Ml,         multiply,      "in" STD_SUP_3 STD_RIGHT_ARROW "m" STD_litre,                "in" STD_SUP_3 STD_RIGHT_ARROW                              ),</v>
       </c>
-      <c r="I37" s="53">
+      <c r="I37" s="52">
         <f>VLOOKUP(A37,Factors!D:G,4,0)</f>
         <v>16.387063999999999</v>
       </c>
-      <c r="J37" s="53" t="str">
+      <c r="J37" s="52" t="str">
         <f t="shared" si="9"/>
         <v>1.638706400000000000000000000000000000000000000000000000e+01</v>
       </c>
-      <c r="K37" s="56" t="str">
+      <c r="K37" s="55" t="str">
         <f>VLOOKUP(A37,Factors!D:N,11,0)</f>
         <v>In3Ml</v>
       </c>
@@ -3834,22 +3890,22 @@
       <c r="B38" s="44" t="s">
         <v>195</v>
       </c>
-      <c r="C38" s="92" t="s">
+      <c r="C38" s="91" t="s">
         <v>70</v>
       </c>
       <c r="D38" s="40" t="str">
         <f>VLOOKUP(A38,Factors!D:K,8,0)</f>
         <v>constFactorFt3Gluk</v>
       </c>
-      <c r="E38" s="53" t="str">
+      <c r="E38" s="52" t="str">
         <f>VLOOKUP(A38,Factors!D:N,10,0)</f>
         <v>multiply</v>
       </c>
-      <c r="F38" s="55" t="str">
+      <c r="F38" s="54" t="str">
         <f t="shared" si="6"/>
         <v>"ft" STD_SUP_3 STD_RIGHT_ARROW "gal" STD_UK</v>
       </c>
-      <c r="G38" s="55" t="str">
+      <c r="G38" s="54" t="str">
         <f t="shared" si="7"/>
         <v>"ft" STD_SUP_3 STD_RIGHT_ARROW</v>
       </c>
@@ -3857,15 +3913,15 @@
         <f t="shared" si="8"/>
         <v>/* NNNN */  UNIT_CONV(constFactorFt3Gluk,       multiply,      "ft" STD_SUP_3 STD_RIGHT_ARROW "gal" STD_UK,                 "ft" STD_SUP_3 STD_RIGHT_ARROW                              ),</v>
       </c>
-      <c r="I38" s="53">
+      <c r="I38" s="52">
         <f>VLOOKUP(A38,Factors!D:G,4,0)</f>
         <v>6.2288354590428261</v>
       </c>
-      <c r="J38" s="53" t="str">
+      <c r="J38" s="52" t="str">
         <f t="shared" si="9"/>
         <v>6.228835459042830000000000000000000000000000000000000000e+00</v>
       </c>
-      <c r="K38" s="56" t="str">
+      <c r="K38" s="55" t="str">
         <f>VLOOKUP(A38,Factors!D:N,11,0)</f>
         <v>Ft3Gluk</v>
       </c>
@@ -3885,22 +3941,22 @@
       <c r="B39" s="44" t="s">
         <v>196</v>
       </c>
-      <c r="C39" s="92" t="s">
+      <c r="C39" s="91" t="s">
         <v>70</v>
       </c>
       <c r="D39" s="40" t="str">
         <f>VLOOKUP(A39,Factors!D:K,8,0)</f>
         <v>constFactorGlukFt3</v>
       </c>
-      <c r="E39" s="53" t="str">
+      <c r="E39" s="52" t="str">
         <f>VLOOKUP(A39,Factors!D:N,10,0)</f>
         <v xml:space="preserve">  divide</v>
       </c>
-      <c r="F39" s="55" t="str">
+      <c r="F39" s="54" t="str">
         <f t="shared" si="6"/>
         <v>"gal" STD_UK STD_RIGHT_ARROW "ft" STD_SUP_3</v>
       </c>
-      <c r="G39" s="55" t="str">
+      <c r="G39" s="54" t="str">
         <f t="shared" si="7"/>
         <v>"gal" STD_UK STD_RIGHT_ARROW</v>
       </c>
@@ -3908,15 +3964,15 @@
         <f t="shared" si="8"/>
         <v>/* NNNN */  UNIT_CONV(constFactorGlukFt3,         divide,      "gal" STD_UK STD_RIGHT_ARROW "ft" STD_SUP_3,                 "gal" STD_UK STD_RIGHT_ARROW                                ),</v>
       </c>
-      <c r="I39" s="53">
+      <c r="I39" s="52">
         <f>VLOOKUP(A39,Factors!D:G,4,0)</f>
         <v>6.2288354590428261</v>
       </c>
-      <c r="J39" s="53" t="str">
+      <c r="J39" s="52" t="str">
         <f t="shared" si="9"/>
         <v>6.228835459042830000000000000000000000000000000000000000e+00</v>
       </c>
-      <c r="K39" s="56" t="str">
+      <c r="K39" s="55" t="str">
         <f>VLOOKUP(A39,Factors!D:N,11,0)</f>
         <v>Ft3Gluk</v>
       </c>
@@ -3936,47 +3992,47 @@
       <c r="B40" s="44" t="s">
         <v>197</v>
       </c>
-      <c r="C40" s="92" t="s">
+      <c r="C40" s="91" t="s">
         <v>70</v>
       </c>
       <c r="D40" s="40" t="str">
         <f>VLOOKUP(A40,Factors!D:K,8,0)</f>
         <v>constFactorLFt3</v>
       </c>
-      <c r="E40" s="53" t="str">
+      <c r="E40" s="52" t="str">
         <f>VLOOKUP(A40,Factors!D:N,10,0)</f>
         <v xml:space="preserve">  divide</v>
       </c>
-      <c r="F40" s="55" t="str">
-        <f t="shared" si="6"/>
+      <c r="F40" s="54" t="str">
+        <f t="shared" ref="F40:F43" si="12" xml:space="preserve"> VLOOKUP(A40,stdform,2,0)</f>
         <v>STD_litre STD_RIGHT_ARROW "ft" STD_SUP_3</v>
       </c>
-      <c r="G40" s="55" t="str">
-        <f t="shared" si="7"/>
+      <c r="G40" s="54" t="str">
+        <f t="shared" ref="G40:G43" si="13">MID(F40,1,SEARCH("STD_RIGHT_ARROW",F40)-2)&amp;" STD_RIGHT_ARROW"</f>
         <v>STD_litre STD_RIGHT_ARROW</v>
       </c>
       <c r="H40" s="30" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" ref="H40:H43" si="14">"/* NNNN */  UNIT_CONV("&amp;D40&amp;","&amp;REPT(CHAR(32),21-LEN(D40))&amp;"    "&amp;E40&amp;",      "&amp;F40&amp;","&amp;REPT(CHAR(32),60-LEN(F40))&amp;G40&amp;REPT(CHAR(32),60-LEN(G40))&amp;"),"</f>
         <v>/* NNNN */  UNIT_CONV(constFactorLFt3,            divide,      STD_litre STD_RIGHT_ARROW "ft" STD_SUP_3,                    STD_litre STD_RIGHT_ARROW                                   ),</v>
       </c>
-      <c r="I40" s="53">
+      <c r="I40" s="52">
         <f>VLOOKUP(A40,Factors!D:G,4,0)</f>
         <v>28.316846592000001</v>
       </c>
-      <c r="J40" s="53" t="str">
-        <f t="shared" si="9"/>
+      <c r="J40" s="52" t="str">
+        <f t="shared" ref="J40:J43" si="15">SUBSTITUTE(TEXT(I40,"0.000000000000000000000000000000000000000000000000000000E+00"),"E","e")</f>
         <v>2.831684659200000000000000000000000000000000000000000000e+01</v>
       </c>
-      <c r="K40" s="56" t="str">
+      <c r="K40" s="55" t="str">
         <f>VLOOKUP(A40,Factors!D:N,11,0)</f>
         <v>Ft3L</v>
       </c>
       <c r="L40" s="31" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" ref="L40:L43" si="16">IF(E40="multiply","  generateConstantArray("&amp;CHAR(34)&amp;K40&amp;CHAR(34)&amp;","&amp;REPT(CHAR(32),14-LEN(K40))&amp;CHAR(34)&amp;"+"&amp;J40&amp;CHAR(34)&amp;");","")</f>
         <v/>
       </c>
       <c r="N40" s="41" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" ref="N40:N43" si="17">"    ["&amp;D40&amp;"] = "&amp;CHAR(38)&amp;"const_"&amp;K40&amp;","</f>
         <v xml:space="preserve">    [constFactorLFt3] = &amp;const_Ft3L,</v>
       </c>
     </row>
@@ -3987,47 +4043,47 @@
       <c r="B41" s="44" t="s">
         <v>198</v>
       </c>
-      <c r="C41" s="92" t="s">
+      <c r="C41" s="91" t="s">
         <v>70</v>
       </c>
       <c r="D41" s="40" t="str">
         <f>VLOOKUP(A41,Factors!D:K,8,0)</f>
         <v>constFactorFt3L</v>
       </c>
-      <c r="E41" s="53" t="str">
+      <c r="E41" s="52" t="str">
         <f>VLOOKUP(A41,Factors!D:N,10,0)</f>
         <v>multiply</v>
       </c>
-      <c r="F41" s="55" t="str">
-        <f t="shared" si="6"/>
+      <c r="F41" s="54" t="str">
+        <f t="shared" si="12"/>
         <v>"ft" STD_SUP_3 STD_RIGHT_ARROW STD_litre</v>
       </c>
-      <c r="G41" s="55" t="str">
-        <f t="shared" si="7"/>
+      <c r="G41" s="54" t="str">
+        <f t="shared" si="13"/>
         <v>"ft" STD_SUP_3 STD_RIGHT_ARROW</v>
       </c>
       <c r="H41" s="30" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="14"/>
         <v>/* NNNN */  UNIT_CONV(constFactorFt3L,          multiply,      "ft" STD_SUP_3 STD_RIGHT_ARROW STD_litre,                    "ft" STD_SUP_3 STD_RIGHT_ARROW                              ),</v>
       </c>
-      <c r="I41" s="53">
+      <c r="I41" s="52">
         <f>VLOOKUP(A41,Factors!D:G,4,0)</f>
         <v>28.316846592000001</v>
       </c>
-      <c r="J41" s="53" t="str">
-        <f t="shared" si="9"/>
+      <c r="J41" s="52" t="str">
+        <f t="shared" si="15"/>
         <v>2.831684659200000000000000000000000000000000000000000000e+01</v>
       </c>
-      <c r="K41" s="56" t="str">
+      <c r="K41" s="55" t="str">
         <f>VLOOKUP(A41,Factors!D:N,11,0)</f>
         <v>Ft3L</v>
       </c>
       <c r="L41" s="31" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="16"/>
         <v xml:space="preserve">  generateConstantArray("Ft3L",          "+2.831684659200000000000000000000000000000000000000000000e+01");</v>
       </c>
       <c r="N41" s="41" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="17"/>
         <v xml:space="preserve">    [constFactorFt3L] = &amp;const_Ft3L,</v>
       </c>
     </row>
@@ -4038,47 +4094,47 @@
       <c r="B42" s="44" t="s">
         <v>199</v>
       </c>
-      <c r="C42" s="92" t="s">
+      <c r="C42" s="91" t="s">
         <v>70</v>
       </c>
       <c r="D42" s="40" t="str">
         <f>VLOOKUP(A42,Factors!D:K,8,0)</f>
         <v>constFactorLQtus</v>
       </c>
-      <c r="E42" s="53" t="str">
+      <c r="E42" s="52" t="str">
         <f>VLOOKUP(A42,Factors!D:N,10,0)</f>
         <v>multiply</v>
       </c>
-      <c r="F42" s="55" t="str">
-        <f t="shared" si="6"/>
+      <c r="F42" s="54" t="str">
+        <f t="shared" si="12"/>
         <v>STD_litre STD_RIGHT_ARROW "qt" STD_US</v>
       </c>
-      <c r="G42" s="55" t="str">
-        <f t="shared" si="7"/>
+      <c r="G42" s="54" t="str">
+        <f t="shared" si="13"/>
         <v>STD_litre STD_RIGHT_ARROW</v>
       </c>
       <c r="H42" s="30" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="14"/>
         <v>/* NNNN */  UNIT_CONV(constFactorLQtus,         multiply,      STD_litre STD_RIGHT_ARROW "qt" STD_US,                       STD_litre STD_RIGHT_ARROW                                   ),</v>
       </c>
-      <c r="I42" s="53">
+      <c r="I42" s="52">
         <f>VLOOKUP(A42,Factors!D:G,4,0)</f>
         <v>1.0566882094325938</v>
       </c>
-      <c r="J42" s="53" t="str">
-        <f t="shared" si="9"/>
+      <c r="J42" s="52" t="str">
+        <f t="shared" si="15"/>
         <v>1.056688209432590000000000000000000000000000000000000000e+00</v>
       </c>
-      <c r="K42" s="56" t="str">
+      <c r="K42" s="55" t="str">
         <f>VLOOKUP(A42,Factors!D:N,11,0)</f>
         <v>LQtus</v>
       </c>
       <c r="L42" s="31" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="16"/>
         <v xml:space="preserve">  generateConstantArray("LQtus",         "+1.056688209432590000000000000000000000000000000000000000e+00");</v>
       </c>
       <c r="N42" s="41" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="17"/>
         <v xml:space="preserve">    [constFactorLQtus] = &amp;const_LQtus,</v>
       </c>
     </row>
@@ -4089,75 +4145,271 @@
       <c r="B43" s="44" t="s">
         <v>200</v>
       </c>
-      <c r="C43" s="92" t="s">
+      <c r="C43" s="91" t="s">
         <v>70</v>
       </c>
       <c r="D43" s="40" t="str">
         <f>VLOOKUP(A43,Factors!D:K,8,0)</f>
         <v>constFactorQtusL</v>
       </c>
-      <c r="E43" s="53" t="str">
+      <c r="E43" s="52" t="str">
         <f>VLOOKUP(A43,Factors!D:N,10,0)</f>
         <v xml:space="preserve">  divide</v>
       </c>
-      <c r="F43" s="55" t="str">
-        <f t="shared" si="0"/>
+      <c r="F43" s="54" t="str">
+        <f t="shared" si="12"/>
         <v>"qt" STD_US STD_RIGHT_ARROW STD_litre</v>
       </c>
-      <c r="G43" s="55" t="str">
-        <f t="shared" si="1"/>
+      <c r="G43" s="54" t="str">
+        <f t="shared" si="13"/>
         <v>"qt" STD_US STD_RIGHT_ARROW</v>
       </c>
       <c r="H43" s="30" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="14"/>
         <v>/* NNNN */  UNIT_CONV(constFactorQtusL,           divide,      "qt" STD_US STD_RIGHT_ARROW STD_litre,                       "qt" STD_US STD_RIGHT_ARROW                                 ),</v>
       </c>
-      <c r="I43" s="53">
+      <c r="I43" s="52">
         <f>VLOOKUP(A43,Factors!D:G,4,0)</f>
         <v>1.0566882094325938</v>
       </c>
-      <c r="J43" s="53" t="str">
-        <f t="shared" si="3"/>
+      <c r="J43" s="52" t="str">
+        <f t="shared" si="15"/>
         <v>1.056688209432590000000000000000000000000000000000000000e+00</v>
       </c>
-      <c r="K43" s="56" t="str">
+      <c r="K43" s="55" t="str">
         <f>VLOOKUP(A43,Factors!D:N,11,0)</f>
         <v>LQtus</v>
       </c>
       <c r="L43" s="31" t="str">
+        <f t="shared" si="16"/>
+        <v/>
+      </c>
+      <c r="N43" s="41" t="str">
+        <f t="shared" si="17"/>
+        <v xml:space="preserve">    [constFactorQtusL] = &amp;const_LQtus,</v>
+      </c>
+    </row>
+    <row r="44" spans="1:14">
+      <c r="A44" s="100" t="s">
+        <v>262</v>
+      </c>
+      <c r="B44" s="44"/>
+      <c r="C44" s="91" t="s">
+        <v>70</v>
+      </c>
+      <c r="D44" s="40" t="str">
+        <f>VLOOKUP(A44,Factors!D:K,8,0)</f>
+        <v>constFactorGlukFzuk</v>
+      </c>
+      <c r="E44" s="52" t="str">
+        <f>VLOOKUP(A44,Factors!D:N,10,0)</f>
+        <v>multiply</v>
+      </c>
+      <c r="F44" s="54" t="str">
+        <f t="shared" si="6"/>
+        <v>"gal" STD_UK STD_RIGHT_ARROW "floz" STD_UK</v>
+      </c>
+      <c r="G44" s="54" t="str">
+        <f t="shared" si="7"/>
+        <v>"gal" STD_UK STD_RIGHT_ARROW</v>
+      </c>
+      <c r="H44" s="30" t="str">
+        <f t="shared" si="8"/>
+        <v>/* NNNN */  UNIT_CONV(constFactorGlukFzuk,      multiply,      "gal" STD_UK STD_RIGHT_ARROW "floz" STD_UK,                  "gal" STD_UK STD_RIGHT_ARROW                                ),</v>
+      </c>
+      <c r="I44" s="52">
+        <f>VLOOKUP(A44,Factors!D:G,4,0)</f>
+        <v>160</v>
+      </c>
+      <c r="J44" s="52" t="str">
+        <f t="shared" si="9"/>
+        <v>1.600000000000000000000000000000000000000000000000000000e+02</v>
+      </c>
+      <c r="K44" s="55" t="str">
+        <f>VLOOKUP(A44,Factors!D:N,11,0)</f>
+        <v>GlukFzuk</v>
+      </c>
+      <c r="L44" s="31" t="str">
+        <f t="shared" si="10"/>
+        <v xml:space="preserve">  generateConstantArray("GlukFzuk",      "+1.600000000000000000000000000000000000000000000000000000e+02");</v>
+      </c>
+      <c r="N44" s="41" t="str">
+        <f t="shared" si="11"/>
+        <v xml:space="preserve">    [constFactorGlukFzuk] = &amp;const_GlukFzuk,</v>
+      </c>
+    </row>
+    <row r="45" spans="1:14">
+      <c r="A45" s="100" t="s">
+        <v>263</v>
+      </c>
+      <c r="B45" s="44"/>
+      <c r="C45" s="91" t="s">
+        <v>70</v>
+      </c>
+      <c r="D45" s="40" t="str">
+        <f>VLOOKUP(A45,Factors!D:K,8,0)</f>
+        <v>constFactorFzukGluk</v>
+      </c>
+      <c r="E45" s="52" t="str">
+        <f>VLOOKUP(A45,Factors!D:N,10,0)</f>
+        <v xml:space="preserve">  divide</v>
+      </c>
+      <c r="F45" s="54" t="str">
+        <f t="shared" si="6"/>
+        <v>"floz" STD_UK STD_RIGHT_ARROW "gal" STD_UK</v>
+      </c>
+      <c r="G45" s="54" t="str">
+        <f t="shared" si="7"/>
+        <v>"floz" STD_UK STD_RIGHT_ARROW</v>
+      </c>
+      <c r="H45" s="30" t="str">
+        <f t="shared" si="8"/>
+        <v>/* NNNN */  UNIT_CONV(constFactorFzukGluk,        divide,      "floz" STD_UK STD_RIGHT_ARROW "gal" STD_UK,                  "floz" STD_UK STD_RIGHT_ARROW                               ),</v>
+      </c>
+      <c r="I45" s="52">
+        <f>VLOOKUP(A45,Factors!D:G,4,0)</f>
+        <v>160</v>
+      </c>
+      <c r="J45" s="52" t="str">
+        <f t="shared" si="9"/>
+        <v>1.600000000000000000000000000000000000000000000000000000e+02</v>
+      </c>
+      <c r="K45" s="55" t="str">
+        <f>VLOOKUP(A45,Factors!D:N,11,0)</f>
+        <v>GlukFzuk</v>
+      </c>
+      <c r="L45" s="31" t="str">
+        <f t="shared" si="10"/>
+        <v/>
+      </c>
+      <c r="N45" s="41" t="str">
+        <f t="shared" si="11"/>
+        <v xml:space="preserve">    [constFactorFzukGluk] = &amp;const_GlukFzuk,</v>
+      </c>
+    </row>
+    <row r="46" spans="1:14">
+      <c r="A46" s="100" t="s">
+        <v>264</v>
+      </c>
+      <c r="B46" s="44"/>
+      <c r="C46" s="91" t="s">
+        <v>70</v>
+      </c>
+      <c r="D46" s="40" t="str">
+        <f>VLOOKUP(A46,Factors!D:K,8,0)</f>
+        <v>constFactorGlusFzus</v>
+      </c>
+      <c r="E46" s="52" t="str">
+        <f>VLOOKUP(A46,Factors!D:N,10,0)</f>
+        <v>multiply</v>
+      </c>
+      <c r="F46" s="54" t="str">
+        <f t="shared" si="6"/>
+        <v>"gal" STD_US STD_RIGHT_ARROW "floz" STD_US</v>
+      </c>
+      <c r="G46" s="54" t="str">
+        <f t="shared" si="7"/>
+        <v>"gal" STD_US STD_RIGHT_ARROW</v>
+      </c>
+      <c r="H46" s="30" t="str">
+        <f t="shared" si="8"/>
+        <v>/* NNNN */  UNIT_CONV(constFactorGlusFzus,      multiply,      "gal" STD_US STD_RIGHT_ARROW "floz" STD_US,                  "gal" STD_US STD_RIGHT_ARROW                                ),</v>
+      </c>
+      <c r="I46" s="52">
+        <f>VLOOKUP(A46,Factors!D:G,4,0)</f>
+        <v>128</v>
+      </c>
+      <c r="J46" s="52" t="str">
+        <f t="shared" si="9"/>
+        <v>1.280000000000000000000000000000000000000000000000000000e+02</v>
+      </c>
+      <c r="K46" s="55" t="str">
+        <f>VLOOKUP(A46,Factors!D:N,11,0)</f>
+        <v>GlusFzus</v>
+      </c>
+      <c r="L46" s="31" t="str">
+        <f t="shared" si="10"/>
+        <v xml:space="preserve">  generateConstantArray("GlusFzus",      "+1.280000000000000000000000000000000000000000000000000000e+02");</v>
+      </c>
+      <c r="N46" s="41" t="str">
+        <f t="shared" si="11"/>
+        <v xml:space="preserve">    [constFactorGlusFzus] = &amp;const_GlusFzus,</v>
+      </c>
+    </row>
+    <row r="47" spans="1:14">
+      <c r="A47" s="100" t="s">
+        <v>265</v>
+      </c>
+      <c r="B47" s="44"/>
+      <c r="C47" s="91" t="s">
+        <v>70</v>
+      </c>
+      <c r="D47" s="40" t="str">
+        <f>VLOOKUP(A47,Factors!D:K,8,0)</f>
+        <v>constFactorFzusGlus</v>
+      </c>
+      <c r="E47" s="52" t="str">
+        <f>VLOOKUP(A47,Factors!D:N,10,0)</f>
+        <v xml:space="preserve">  divide</v>
+      </c>
+      <c r="F47" s="54" t="str">
+        <f t="shared" si="0"/>
+        <v>"floz" STD_US STD_RIGHT_ARROW "gal" STD_US</v>
+      </c>
+      <c r="G47" s="54" t="str">
+        <f t="shared" si="1"/>
+        <v>"floz" STD_US STD_RIGHT_ARROW</v>
+      </c>
+      <c r="H47" s="30" t="str">
+        <f t="shared" si="2"/>
+        <v>/* NNNN */  UNIT_CONV(constFactorFzusGlus,        divide,      "floz" STD_US STD_RIGHT_ARROW "gal" STD_US,                  "floz" STD_US STD_RIGHT_ARROW                               ),</v>
+      </c>
+      <c r="I47" s="52">
+        <f>VLOOKUP(A47,Factors!D:G,4,0)</f>
+        <v>128</v>
+      </c>
+      <c r="J47" s="52" t="str">
+        <f t="shared" si="3"/>
+        <v>1.280000000000000000000000000000000000000000000000000000e+02</v>
+      </c>
+      <c r="K47" s="55" t="str">
+        <f>VLOOKUP(A47,Factors!D:N,11,0)</f>
+        <v>GlusFzus</v>
+      </c>
+      <c r="L47" s="31" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="N43" s="41" t="str">
+      <c r="N47" s="41" t="str">
         <f t="shared" si="5"/>
-        <v xml:space="preserve">    [constFactorQtusL] = &amp;const_LQtus,</v>
-      </c>
-    </row>
-    <row r="45" spans="1:14">
-      <c r="A45" s="4" t="s">
+        <v xml:space="preserve">    [constFactorFzusGlus] = &amp;const_GlusFzus,</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3">
+      <c r="A49" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="B45" s="5" t="s">
+      <c r="B49" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="C45" s="3" t="s">
+      <c r="C49" s="3" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="46" spans="1:14">
-      <c r="A46" s="4" t="s">
+    <row r="50" spans="1:3">
+      <c r="A50" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="B46" s="5" t="s">
+      <c r="B50" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="C46" s="3" t="s">
+      <c r="C50" s="3" t="s">
         <v>71</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:B47">
-    <sortCondition ref="A4:A47"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:B51">
+    <sortCondition ref="A4:A51"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
@@ -4166,7 +4418,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0EAAB5F5-5A0E-F540-8CD7-68987B744E5F}">
-  <dimension ref="A1:R69"/>
+  <dimension ref="A1:R73"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="12.6640625" bestFit="1" customWidth="1"/>
@@ -4182,17 +4434,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="17" thickBot="1">
-      <c r="F1" s="69" t="s">
+      <c r="F1" s="68" t="s">
         <v>218</v>
       </c>
     </row>
     <row r="2" spans="1:18">
-      <c r="F2" s="60" t="s">
+      <c r="F2" s="59" t="s">
         <v>215</v>
       </c>
     </row>
     <row r="3" spans="1:18" ht="17" thickBot="1">
-      <c r="F3" s="61" t="s">
+      <c r="F3" s="60" t="s">
         <v>216</v>
       </c>
     </row>
@@ -4214,24 +4466,24 @@
       </c>
     </row>
     <row r="6" spans="1:18">
-      <c r="C6" s="70" t="s">
+      <c r="C6" s="69" t="s">
         <v>173</v>
       </c>
-      <c r="D6" s="71"/>
+      <c r="D6" s="70"/>
       <c r="E6" s="3" t="s">
         <v>174</v>
       </c>
-      <c r="F6" s="74">
+      <c r="F6" s="73">
         <v>3785.4117839999999</v>
       </c>
-      <c r="G6" s="58" t="s">
+      <c r="G6" s="57" t="s">
         <v>229</v>
       </c>
-      <c r="H6" s="82">
+      <c r="H6" s="81">
         <f>231 * 0.0254^3 * 1000000</f>
         <v>3785.4117839999999</v>
       </c>
-      <c r="I6" s="83">
+      <c r="I6" s="82">
         <f>H6/$H$12</f>
         <v>768</v>
       </c>
@@ -4251,27 +4503,27 @@
       <c r="Q6" s="25"/>
     </row>
     <row r="7" spans="1:18">
-      <c r="C7" s="72" t="s">
+      <c r="C7" s="71" t="s">
         <v>111</v>
       </c>
-      <c r="D7" s="77" t="s">
+      <c r="D7" s="76" t="s">
         <v>131</v>
       </c>
-      <c r="E7" s="78" t="s">
+      <c r="E7" s="77" t="s">
         <v>140</v>
       </c>
-      <c r="F7" s="95">
+      <c r="F7" s="94">
         <f>H7</f>
         <v>946.35294599999997</v>
       </c>
-      <c r="G7" s="58" t="s">
+      <c r="G7" s="57" t="s">
         <v>228</v>
       </c>
-      <c r="H7" s="84">
+      <c r="H7" s="83">
         <f>(231*0.0254^3/128*1000000)/2*32*2</f>
         <v>946.35294599999997</v>
       </c>
-      <c r="I7" s="83">
+      <c r="I7" s="82">
         <f t="shared" ref="I7:I11" si="2">H7/$H$12</f>
         <v>192</v>
       </c>
@@ -4292,26 +4544,26 @@
       <c r="R7" s="25"/>
     </row>
     <row r="8" spans="1:18">
-      <c r="C8" s="72" t="s">
+      <c r="C8" s="71" t="s">
         <v>114</v>
       </c>
-      <c r="D8" s="79" t="s">
+      <c r="D8" s="78" t="s">
         <v>142</v>
       </c>
-      <c r="E8" s="78" t="s">
+      <c r="E8" s="77" t="s">
         <v>141</v>
       </c>
-      <c r="F8" s="59">
+      <c r="F8" s="58">
         <v>473.17647299999999</v>
       </c>
-      <c r="G8" s="58" t="s">
+      <c r="G8" s="57" t="s">
         <v>227</v>
       </c>
-      <c r="H8" s="84">
+      <c r="H8" s="83">
         <f>(231 * 0.0254^3 / 128 * 1000000) / 2 * 32</f>
         <v>473.17647299999999</v>
       </c>
-      <c r="I8" s="83">
+      <c r="I8" s="82">
         <f t="shared" si="2"/>
         <v>96</v>
       </c>
@@ -4331,26 +4583,26 @@
       <c r="Q8" s="25"/>
     </row>
     <row r="9" spans="1:18">
-      <c r="C9" s="72" t="s">
+      <c r="C9" s="71" t="s">
         <v>104</v>
       </c>
-      <c r="D9" s="79" t="s">
+      <c r="D9" s="78" t="s">
         <v>139</v>
       </c>
-      <c r="E9" s="78" t="s">
+      <c r="E9" s="77" t="s">
         <v>138</v>
       </c>
-      <c r="F9" s="59">
+      <c r="F9" s="58">
         <v>236.58823649999999</v>
       </c>
-      <c r="G9" s="58" t="s">
+      <c r="G9" s="57" t="s">
         <v>230</v>
       </c>
-      <c r="H9" s="85">
+      <c r="H9" s="84">
         <f>(231*0.0254^3/128*1000000)/2*32/2</f>
         <v>236.58823649999999</v>
       </c>
-      <c r="I9" s="83">
+      <c r="I9" s="82">
         <f t="shared" si="2"/>
         <v>48</v>
       </c>
@@ -4370,27 +4622,27 @@
       <c r="Q9" s="25"/>
     </row>
     <row r="10" spans="1:18">
-      <c r="A10" s="52" t="s">
+      <c r="A10" s="51" t="s">
         <v>111</v>
       </c>
-      <c r="C10" s="70" t="s">
+      <c r="C10" s="69" t="s">
         <v>95</v>
       </c>
-      <c r="D10" s="71"/>
+      <c r="D10" s="70"/>
       <c r="E10" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="F10" s="74">
+      <c r="F10" s="73">
         <v>29.573529562499999</v>
       </c>
-      <c r="G10" s="58" t="s">
+      <c r="G10" s="57" t="s">
         <v>214</v>
       </c>
-      <c r="H10" s="82">
+      <c r="H10" s="81">
         <f>231 * 0.0254^3 / 128 * 1000000</f>
         <v>29.573529562499999</v>
       </c>
-      <c r="I10" s="96">
+      <c r="I10" s="95">
         <f t="shared" si="2"/>
         <v>6</v>
       </c>
@@ -4409,33 +4661,33 @@
       <c r="P10" s="26"/>
     </row>
     <row r="11" spans="1:18">
-      <c r="C11" s="72" t="s">
+      <c r="C11" s="71" t="s">
         <v>101</v>
       </c>
-      <c r="D11" s="79" t="s">
+      <c r="D11" s="78" t="s">
         <v>137</v>
       </c>
-      <c r="E11" s="78" t="s">
+      <c r="E11" s="77" t="s">
         <v>136</v>
       </c>
-      <c r="F11" s="59">
+      <c r="F11" s="58">
         <v>14.78676478125</v>
       </c>
       <c r="G11" s="25" t="s">
         <v>231</v>
       </c>
-      <c r="H11" s="86">
+      <c r="H11" s="85">
         <f>(231 * 0.0254^3 / 128 * 1000000) / 2</f>
         <v>14.78676478125</v>
       </c>
-      <c r="I11" s="83">
+      <c r="I11" s="82">
         <f t="shared" si="2"/>
         <v>3</v>
       </c>
       <c r="J11" t="s">
         <v>255</v>
       </c>
-      <c r="K11" s="93">
+      <c r="K11" s="92">
         <f t="shared" si="0"/>
         <v>14.78676478125</v>
       </c>
@@ -4447,33 +4699,33 @@
       <c r="P11" s="26"/>
     </row>
     <row r="12" spans="1:18">
-      <c r="C12" s="72" t="s">
+      <c r="C12" s="71" t="s">
         <v>96</v>
       </c>
-      <c r="D12" s="79" t="s">
+      <c r="D12" s="78" t="s">
         <v>135</v>
       </c>
-      <c r="E12" s="78" t="s">
+      <c r="E12" s="77" t="s">
         <v>134</v>
       </c>
-      <c r="F12" s="59">
+      <c r="F12" s="58">
         <v>4.9289215937500002</v>
       </c>
       <c r="G12" s="25" t="s">
         <v>232</v>
       </c>
-      <c r="H12" s="86">
+      <c r="H12" s="85">
         <f>(231 * 0.0254^3 / 128 * 1000000) / 2 / 3</f>
         <v>4.9289215937500002</v>
       </c>
-      <c r="I12" s="83">
+      <c r="I12" s="82">
         <f>H12/$H$12</f>
         <v>1</v>
       </c>
       <c r="J12" t="s">
         <v>255</v>
       </c>
-      <c r="K12" s="93">
+      <c r="K12" s="92">
         <f>$H$6/$I$6*I12</f>
         <v>4.9289215937500002</v>
       </c>
@@ -4485,25 +4737,25 @@
       <c r="P12" s="26"/>
     </row>
     <row r="13" spans="1:18">
-      <c r="C13" s="70" t="s">
+      <c r="C13" s="69" t="s">
         <v>176</v>
       </c>
-      <c r="D13" s="71"/>
+      <c r="D13" s="70"/>
       <c r="E13" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="F13" s="95">
+      <c r="F13" s="94">
         <f>H13</f>
         <v>4546.09</v>
       </c>
-      <c r="G13" s="58" t="s">
+      <c r="G13" s="57" t="s">
         <v>241</v>
       </c>
-      <c r="H13" s="82">
+      <c r="H13" s="81">
         <f>0.00454609 * 1000000</f>
         <v>4546.09</v>
       </c>
-      <c r="I13" s="87">
+      <c r="I13" s="86">
         <f t="shared" ref="I13:I19" si="3">H13/$H$19</f>
         <v>768</v>
       </c>
@@ -4523,27 +4775,27 @@
       <c r="Q13" s="25"/>
     </row>
     <row r="14" spans="1:18">
-      <c r="A14" s="52"/>
-      <c r="C14" s="73" t="s">
+      <c r="A14" s="51"/>
+      <c r="C14" s="72" t="s">
         <v>89</v>
       </c>
-      <c r="D14" s="80" t="s">
+      <c r="D14" s="79" t="s">
         <v>131</v>
       </c>
-      <c r="E14" s="81" t="s">
+      <c r="E14" s="80" t="s">
         <v>130</v>
       </c>
-      <c r="F14" s="59">
+      <c r="F14" s="58">
         <v>1136.5225</v>
       </c>
-      <c r="G14" s="58" t="s">
+      <c r="G14" s="57" t="s">
         <v>213</v>
       </c>
-      <c r="H14" s="82">
+      <c r="H14" s="81">
         <f>0.00454609 / 4 * 1000000</f>
         <v>1136.5225</v>
       </c>
-      <c r="I14" s="87">
+      <c r="I14" s="86">
         <f t="shared" si="3"/>
         <v>192</v>
       </c>
@@ -4564,26 +4816,26 @@
       <c r="Q14" s="25"/>
     </row>
     <row r="15" spans="1:18">
-      <c r="A15" s="52"/>
-      <c r="C15" s="72" t="s">
+      <c r="A15" s="51"/>
+      <c r="C15" s="71" t="s">
         <v>92</v>
       </c>
-      <c r="D15" s="79" t="s">
+      <c r="D15" s="78" t="s">
         <v>133</v>
       </c>
-      <c r="E15" s="78" t="s">
+      <c r="E15" s="77" t="s">
         <v>132</v>
       </c>
-      <c r="F15" s="59">
+      <c r="F15" s="58">
         <v>568.26125000000002</v>
       </c>
-      <c r="G15" s="58" t="s">
+      <c r="G15" s="57" t="s">
         <v>242</v>
       </c>
-      <c r="H15" s="82">
+      <c r="H15" s="81">
         <v>568.26125000000002</v>
       </c>
-      <c r="I15" s="87">
+      <c r="I15" s="86">
         <f t="shared" si="3"/>
         <v>96</v>
       </c>
@@ -4604,27 +4856,27 @@
       <c r="Q15" s="28"/>
     </row>
     <row r="16" spans="1:18">
-      <c r="A16" s="52"/>
-      <c r="C16" s="72" t="s">
+      <c r="A16" s="51"/>
+      <c r="C16" s="71" t="s">
         <v>82</v>
       </c>
-      <c r="D16" s="79" t="s">
+      <c r="D16" s="78" t="s">
         <v>129</v>
       </c>
-      <c r="E16" s="78" t="s">
+      <c r="E16" s="77" t="s">
         <v>128</v>
       </c>
-      <c r="F16" s="59">
+      <c r="F16" s="58">
         <v>284.13062500000001</v>
       </c>
-      <c r="G16" s="58" t="s">
+      <c r="G16" s="57" t="s">
         <v>252</v>
       </c>
-      <c r="H16" s="82">
+      <c r="H16" s="81">
         <f>0.00454609 / 16 * 1000000</f>
         <v>284.13062500000001</v>
       </c>
-      <c r="I16" s="87">
+      <c r="I16" s="86">
         <f t="shared" si="3"/>
         <v>48</v>
       </c>
@@ -4645,25 +4897,25 @@
       <c r="Q16" s="28"/>
     </row>
     <row r="17" spans="1:16">
-      <c r="A17" s="52"/>
-      <c r="C17" s="70" t="s">
+      <c r="A17" s="51"/>
+      <c r="C17" s="69" t="s">
         <v>72</v>
       </c>
-      <c r="D17" s="71"/>
+      <c r="D17" s="70"/>
       <c r="E17" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="F17" s="74">
+      <c r="F17" s="73">
         <v>28.413062500000002</v>
       </c>
-      <c r="G17" s="58" t="s">
+      <c r="G17" s="57" t="s">
         <v>240</v>
       </c>
-      <c r="H17" s="82">
+      <c r="H17" s="81">
         <f xml:space="preserve"> 0.00454609 / 160 * 1000000</f>
         <v>28.413062500000002</v>
       </c>
-      <c r="I17" s="97">
+      <c r="I17" s="96">
         <f t="shared" si="3"/>
         <v>4.8</v>
       </c>
@@ -4682,29 +4934,29 @@
       <c r="P17" s="26"/>
     </row>
     <row r="18" spans="1:16">
-      <c r="A18" s="52" t="s">
+      <c r="A18" s="51" t="s">
         <v>201</v>
       </c>
-      <c r="C18" s="72" t="s">
+      <c r="C18" s="71" t="s">
         <v>79</v>
       </c>
-      <c r="D18" s="79" t="s">
+      <c r="D18" s="78" t="s">
         <v>127</v>
       </c>
-      <c r="E18" s="78" t="s">
+      <c r="E18" s="77" t="s">
         <v>126</v>
       </c>
-      <c r="F18" s="59">
+      <c r="F18" s="58">
         <v>17.758164062500001</v>
       </c>
-      <c r="G18" s="58" t="s">
+      <c r="G18" s="57" t="s">
         <v>253</v>
       </c>
-      <c r="H18" s="88">
+      <c r="H18" s="87">
         <f>568.26125/32</f>
         <v>17.758164062500001</v>
       </c>
-      <c r="I18" s="87">
+      <c r="I18" s="86">
         <f t="shared" si="3"/>
         <v>3</v>
       </c>
@@ -4724,37 +4976,37 @@
       <c r="P18" s="26"/>
     </row>
     <row r="19" spans="1:16">
-      <c r="A19" s="52" t="s">
+      <c r="A19" s="51" t="s">
         <v>207</v>
       </c>
-      <c r="C19" s="72" t="s">
+      <c r="C19" s="71" t="s">
         <v>73</v>
       </c>
-      <c r="D19" s="79" t="s">
+      <c r="D19" s="78" t="s">
         <v>125</v>
       </c>
-      <c r="E19" s="78" t="s">
+      <c r="E19" s="77" t="s">
         <v>124</v>
       </c>
-      <c r="F19" s="75">
+      <c r="F19" s="74">
         <f>H19</f>
         <v>5.9193880208333338</v>
       </c>
-      <c r="G19" s="58" t="s">
+      <c r="G19" s="57" t="s">
         <v>254</v>
       </c>
-      <c r="H19" s="89">
+      <c r="H19" s="88">
         <f>568.26125/96</f>
         <v>5.9193880208333338</v>
       </c>
-      <c r="I19" s="87">
+      <c r="I19" s="86">
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="J19" t="s">
         <v>256</v>
       </c>
-      <c r="K19" s="94">
+      <c r="K19" s="93">
         <f>$H$13/$I$13*I19</f>
         <v>5.9193880208333338</v>
       </c>
@@ -4767,100 +5019,100 @@
       <c r="P19" s="26"/>
     </row>
     <row r="20" spans="1:16">
-      <c r="A20" s="52" t="s">
+      <c r="A20" s="51" t="s">
         <v>208</v>
       </c>
-      <c r="C20" s="70" t="s">
+      <c r="C20" s="69" t="s">
         <v>76</v>
       </c>
-      <c r="D20" s="71" t="s">
+      <c r="D20" s="70" t="s">
         <v>123</v>
       </c>
       <c r="E20" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="F20" s="59">
+      <c r="F20" s="58">
         <v>1</v>
       </c>
-      <c r="G20" s="58" t="s">
+      <c r="G20" s="57" t="s">
         <v>217</v>
       </c>
-      <c r="H20" s="82">
+      <c r="H20" s="81">
         <v>1</v>
       </c>
-      <c r="I20" s="90"/>
+      <c r="I20" s="89"/>
       <c r="M20" s="7"/>
       <c r="P20" s="26"/>
     </row>
     <row r="21" spans="1:16">
-      <c r="C21" s="70" t="s">
+      <c r="C21" s="69" t="s">
         <v>201</v>
       </c>
-      <c r="D21" s="71"/>
+      <c r="D21" s="70"/>
       <c r="E21" s="3"/>
-      <c r="F21" s="59">
+      <c r="F21" s="58">
         <f>2.54^3</f>
         <v>16.387063999999999</v>
       </c>
-      <c r="G21" s="58" t="s">
+      <c r="G21" s="57" t="s">
         <v>247</v>
       </c>
-      <c r="H21" s="82">
+      <c r="H21" s="81">
         <f>2.54^3</f>
         <v>16.387063999999999</v>
       </c>
-      <c r="I21" s="90"/>
+      <c r="I21" s="89"/>
       <c r="J21" s="24"/>
       <c r="K21" s="25"/>
     </row>
     <row r="22" spans="1:16">
-      <c r="C22" s="70" t="s">
+      <c r="C22" s="69" t="s">
         <v>207</v>
       </c>
-      <c r="D22" s="71"/>
+      <c r="D22" s="70"/>
       <c r="E22" s="3"/>
-      <c r="F22" s="76">
+      <c r="F22" s="75">
         <f>(12*2.54)^3</f>
         <v>28316.846592000002</v>
       </c>
-      <c r="G22" s="58" t="s">
+      <c r="G22" s="57" t="s">
         <v>248</v>
       </c>
-      <c r="H22" s="84">
+      <c r="H22" s="83">
         <f>(12*2.54)^3</f>
         <v>28316.846592000002</v>
       </c>
-      <c r="I22" s="90"/>
+      <c r="I22" s="89"/>
       <c r="J22" s="24"/>
       <c r="K22" s="25"/>
     </row>
     <row r="23" spans="1:16">
-      <c r="C23" s="70" t="s">
+      <c r="C23" s="69" t="s">
         <v>208</v>
       </c>
-      <c r="D23" s="71"/>
+      <c r="D23" s="70"/>
       <c r="E23" s="3"/>
-      <c r="F23" s="59">
+      <c r="F23" s="58">
         <v>1000</v>
       </c>
-      <c r="G23" s="58" t="s">
+      <c r="G23" s="57" t="s">
         <v>249</v>
       </c>
-      <c r="H23" s="82"/>
-      <c r="I23" s="90"/>
+      <c r="H23" s="81"/>
+      <c r="I23" s="89"/>
       <c r="J23" s="24"/>
       <c r="K23" s="25"/>
     </row>
     <row r="24" spans="1:16">
-      <c r="C24" s="52"/>
+      <c r="C24" s="51"/>
       <c r="F24" s="34"/>
-      <c r="G24" s="66"/>
+      <c r="G24" s="65"/>
       <c r="J24" s="24"/>
       <c r="K24" s="25"/>
     </row>
     <row r="25" spans="1:16">
       <c r="F25" s="1"/>
-      <c r="H25" s="62">
+      <c r="H25" s="61">
         <f xml:space="preserve"> 568.26125 / 20</f>
         <v>28.413062500000002</v>
       </c>
@@ -4945,7 +5197,7 @@
         <v>3</v>
       </c>
       <c r="F29" s="36">
-        <f t="shared" ref="F29:F69" si="7">H29/I29</f>
+        <f t="shared" ref="F29:F73" si="7">H29/I29</f>
         <v>2.1133764188651875E-3</v>
       </c>
       <c r="G29" s="38">
@@ -6501,15 +6753,15 @@
       </c>
     </row>
     <row r="62" spans="1:14" ht="18">
-      <c r="A62" s="51" t="str">
+      <c r="A62" s="50" t="str">
         <f>MID(D62,5,99)</f>
         <v>MLtoIN3</v>
       </c>
-      <c r="B62" s="52" t="str">
+      <c r="B62" s="51" t="str">
         <f>MID(A62,1,SEARCH("to",A62)-1)</f>
         <v>ML</v>
       </c>
-      <c r="C62" s="52" t="str">
+      <c r="C62" s="51" t="str">
         <f>MID(A62,SEARCH("to",A62)+2,99)</f>
         <v>IN3</v>
       </c>
@@ -6532,15 +6784,15 @@
         <v>1</v>
       </c>
       <c r="I62" s="9">
-        <f t="shared" ref="I62:I69" si="27" xml:space="preserve"> VLOOKUP(C62,units,4,0)</f>
+        <f t="shared" ref="I62:I73" si="27" xml:space="preserve"> VLOOKUP(C62,units,4,0)</f>
         <v>16.387063999999999</v>
       </c>
       <c r="J62" t="str">
-        <f t="shared" ref="J62:J69" si="28">PROPER(B62)&amp;PROPER(C62)</f>
+        <f t="shared" ref="J62:J73" si="28">PROPER(B62)&amp;PROPER(C62)</f>
         <v>MlIn3</v>
       </c>
       <c r="K62" t="str">
-        <f t="shared" ref="K62:K69" si="29">"constFactor"&amp;J62</f>
+        <f t="shared" ref="K62:K73" si="29">"constFactor"&amp;J62</f>
         <v>constFactorMlIn3</v>
       </c>
       <c r="M62" s="38" t="str">
@@ -6553,16 +6805,16 @@
       </c>
     </row>
     <row r="63" spans="1:14" ht="18">
-      <c r="A63" s="51" t="str">
-        <f t="shared" ref="A63:A69" si="30">MID(D63,5,99)</f>
+      <c r="A63" s="50" t="str">
+        <f t="shared" ref="A63:A73" si="30">MID(D63,5,99)</f>
         <v>IN3toML</v>
       </c>
-      <c r="B63" s="52" t="str">
-        <f t="shared" ref="B63:B69" si="31">MID(A63,1,SEARCH("to",A63)-1)</f>
+      <c r="B63" s="51" t="str">
+        <f t="shared" ref="B63:B73" si="31">MID(A63,1,SEARCH("to",A63)-1)</f>
         <v>IN3</v>
       </c>
-      <c r="C63" s="52" t="str">
-        <f t="shared" ref="C63:C69" si="32">MID(A63,SEARCH("to",A63)+2,99)</f>
+      <c r="C63" s="51" t="str">
+        <f t="shared" ref="C63:C73" si="32">MID(A63,SEARCH("to",A63)+2,99)</f>
         <v>ML</v>
       </c>
       <c r="D63" s="47" t="s">
@@ -6580,7 +6832,7 @@
         <v>16.387063999999999</v>
       </c>
       <c r="H63" s="9">
-        <f t="shared" ref="H63:H69" si="33" xml:space="preserve"> VLOOKUP(B63,units,4,0)</f>
+        <f t="shared" ref="H63:H73" si="33" xml:space="preserve"> VLOOKUP(B63,units,4,0)</f>
         <v>16.387063999999999</v>
       </c>
       <c r="I63" s="9">
@@ -6605,15 +6857,15 @@
       </c>
     </row>
     <row r="64" spans="1:14" ht="18">
-      <c r="A64" s="51" t="str">
+      <c r="A64" s="50" t="str">
         <f t="shared" si="30"/>
         <v>FT3toGLUK</v>
       </c>
-      <c r="B64" s="52" t="str">
+      <c r="B64" s="51" t="str">
         <f t="shared" si="31"/>
         <v>FT3</v>
       </c>
-      <c r="C64" s="52" t="str">
+      <c r="C64" s="51" t="str">
         <f t="shared" si="32"/>
         <v>GLUK</v>
       </c>
@@ -6657,15 +6909,15 @@
       </c>
     </row>
     <row r="65" spans="1:14" ht="18">
-      <c r="A65" s="51" t="str">
+      <c r="A65" s="50" t="str">
         <f t="shared" si="30"/>
         <v>GLUKtoFT3</v>
       </c>
-      <c r="B65" s="52" t="str">
+      <c r="B65" s="51" t="str">
         <f t="shared" si="31"/>
         <v>GLUK</v>
       </c>
-      <c r="C65" s="52" t="str">
+      <c r="C65" s="51" t="str">
         <f t="shared" si="32"/>
         <v>FT3</v>
       </c>
@@ -6709,16 +6961,16 @@
       </c>
     </row>
     <row r="66" spans="1:14" ht="18">
-      <c r="A66" s="51" t="str">
-        <f t="shared" si="30"/>
+      <c r="A66" s="50" t="str">
+        <f t="shared" ref="A66:A69" si="34">MID(D66,5,99)</f>
         <v>LtoFT3</v>
       </c>
-      <c r="B66" s="52" t="str">
-        <f t="shared" si="31"/>
+      <c r="B66" s="51" t="str">
+        <f t="shared" ref="B66:B69" si="35">MID(A66,1,SEARCH("to",A66)-1)</f>
         <v>L</v>
       </c>
-      <c r="C66" s="52" t="str">
-        <f t="shared" si="32"/>
+      <c r="C66" s="51" t="str">
+        <f t="shared" ref="C66:C69" si="36">MID(A66,SEARCH("to",A66)+2,99)</f>
         <v>FT3</v>
       </c>
       <c r="D66" s="47" t="s">
@@ -6728,49 +6980,49 @@
         <v>197</v>
       </c>
       <c r="F66" s="36">
-        <f t="shared" si="7"/>
+        <f t="shared" ref="F66:F69" si="37">H66/I66</f>
         <v>3.5314666721488586E-2</v>
       </c>
-      <c r="G66" s="38">
+      <c r="G66" s="39">
         <f>IF(M66="multiply",F66,F67)</f>
         <v>28.316846592000001</v>
       </c>
       <c r="H66" s="9">
-        <f t="shared" si="33"/>
+        <f t="shared" ref="H66:H69" si="38" xml:space="preserve"> VLOOKUP(B66,units,4,0)</f>
         <v>1000</v>
       </c>
       <c r="I66" s="9">
-        <f t="shared" si="27"/>
+        <f t="shared" ref="I66:I69" si="39" xml:space="preserve"> VLOOKUP(C66,units,4,0)</f>
         <v>28316.846592000002</v>
       </c>
       <c r="J66" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" ref="J66:J69" si="40">PROPER(B66)&amp;PROPER(C66)</f>
         <v>LFt3</v>
       </c>
       <c r="K66" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" ref="K66:K69" si="41">"constFactor"&amp;J66</f>
         <v>constFactorLFt3</v>
       </c>
-      <c r="M66" s="38" t="str">
+      <c r="M66" s="39" t="str">
         <f>IF(H66&gt;I66,"multiply","  divide")</f>
         <v xml:space="preserve">  divide</v>
       </c>
-      <c r="N66" s="38" t="str">
+      <c r="N66" s="39" t="str">
         <f>IF(M66="multiply",PROPER(B66)&amp;PROPER(C66),J67)</f>
         <v>Ft3L</v>
       </c>
     </row>
     <row r="67" spans="1:14" ht="18">
-      <c r="A67" s="51" t="str">
-        <f t="shared" si="30"/>
+      <c r="A67" s="50" t="str">
+        <f t="shared" si="34"/>
         <v>FT3toL</v>
       </c>
-      <c r="B67" s="52" t="str">
-        <f t="shared" si="31"/>
+      <c r="B67" s="51" t="str">
+        <f t="shared" si="35"/>
         <v>FT3</v>
       </c>
-      <c r="C67" s="52" t="str">
-        <f t="shared" si="32"/>
+      <c r="C67" s="51" t="str">
+        <f t="shared" si="36"/>
         <v>L</v>
       </c>
       <c r="D67" s="47" t="s">
@@ -6780,49 +7032,49 @@
         <v>198</v>
       </c>
       <c r="F67" s="36">
-        <f t="shared" si="7"/>
+        <f t="shared" si="37"/>
         <v>28.316846592000001</v>
       </c>
-      <c r="G67" s="38">
+      <c r="G67" s="39">
         <f>IF(M67="multiply",F67,F66)</f>
         <v>28.316846592000001</v>
       </c>
       <c r="H67" s="9">
-        <f t="shared" si="33"/>
+        <f t="shared" si="38"/>
         <v>28316.846592000002</v>
       </c>
       <c r="I67" s="9">
-        <f t="shared" si="27"/>
+        <f t="shared" si="39"/>
         <v>1000</v>
       </c>
       <c r="J67" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="40"/>
         <v>Ft3L</v>
       </c>
       <c r="K67" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="41"/>
         <v>constFactorFt3L</v>
       </c>
-      <c r="M67" s="38" t="str">
+      <c r="M67" s="39" t="str">
         <f>IF(M66="multiply","  divide","multiply")</f>
         <v>multiply</v>
       </c>
-      <c r="N67" s="38" t="str">
+      <c r="N67" s="39" t="str">
         <f>IF(M67="multiply",PROPER(B67)&amp;PROPER(C67),J66)</f>
         <v>Ft3L</v>
       </c>
     </row>
     <row r="68" spans="1:14" ht="18">
-      <c r="A68" s="51" t="str">
-        <f t="shared" si="30"/>
+      <c r="A68" s="50" t="str">
+        <f t="shared" si="34"/>
         <v>LtoQTUS</v>
       </c>
-      <c r="B68" s="52" t="str">
-        <f t="shared" si="31"/>
+      <c r="B68" s="51" t="str">
+        <f t="shared" si="35"/>
         <v>L</v>
       </c>
-      <c r="C68" s="52" t="str">
-        <f t="shared" si="32"/>
+      <c r="C68" s="51" t="str">
+        <f t="shared" si="36"/>
         <v>QTUS</v>
       </c>
       <c r="D68" s="47" t="s">
@@ -6832,7 +7084,7 @@
         <v>199</v>
       </c>
       <c r="F68" s="36">
-        <f t="shared" si="7"/>
+        <f t="shared" si="37"/>
         <v>1.0566882094325938</v>
       </c>
       <c r="G68" s="39">
@@ -6840,19 +7092,19 @@
         <v>1.0566882094325938</v>
       </c>
       <c r="H68" s="9">
-        <f t="shared" si="33"/>
+        <f t="shared" si="38"/>
         <v>1000</v>
       </c>
       <c r="I68" s="9">
-        <f t="shared" si="27"/>
+        <f t="shared" si="39"/>
         <v>946.35294599999997</v>
       </c>
       <c r="J68" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="40"/>
         <v>LQtus</v>
       </c>
       <c r="K68" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="41"/>
         <v>constFactorLQtus</v>
       </c>
       <c r="M68" s="39" t="str">
@@ -6864,27 +7116,27 @@
         <v>LQtus</v>
       </c>
     </row>
-    <row r="69" spans="1:14" ht="19" thickBot="1">
-      <c r="A69" s="51" t="str">
-        <f t="shared" si="30"/>
+    <row r="69" spans="1:14" ht="18">
+      <c r="A69" s="50" t="str">
+        <f t="shared" si="34"/>
         <v>QTUStoL</v>
       </c>
-      <c r="B69" s="52" t="str">
-        <f t="shared" si="31"/>
+      <c r="B69" s="51" t="str">
+        <f t="shared" si="35"/>
         <v>QTUS</v>
       </c>
-      <c r="C69" s="52" t="str">
-        <f t="shared" si="32"/>
+      <c r="C69" s="51" t="str">
+        <f t="shared" si="36"/>
         <v>L</v>
       </c>
-      <c r="D69" s="49" t="s">
+      <c r="D69" s="47" t="s">
         <v>192</v>
       </c>
-      <c r="E69" s="50" t="s">
+      <c r="E69" s="48" t="s">
         <v>200</v>
       </c>
       <c r="F69" s="36">
-        <f t="shared" si="7"/>
+        <f t="shared" si="37"/>
         <v>0.94635294599999997</v>
       </c>
       <c r="G69" s="39">
@@ -6892,19 +7144,19 @@
         <v>1.0566882094325938</v>
       </c>
       <c r="H69" s="9">
-        <f t="shared" si="33"/>
+        <f t="shared" si="38"/>
         <v>946.35294599999997</v>
       </c>
       <c r="I69" s="9">
-        <f t="shared" si="27"/>
+        <f t="shared" si="39"/>
         <v>1000</v>
       </c>
       <c r="J69" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="40"/>
         <v>QtusL</v>
       </c>
       <c r="K69" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="41"/>
         <v>constFactorQtusL</v>
       </c>
       <c r="M69" s="39" t="str">
@@ -6914,6 +7166,206 @@
       <c r="N69" s="39" t="str">
         <f>IF(M69="multiply",PROPER(B69)&amp;PROPER(C69),J68)</f>
         <v>LQtus</v>
+      </c>
+    </row>
+    <row r="70" spans="1:14" ht="18">
+      <c r="A70" s="50" t="str">
+        <f t="shared" si="30"/>
+        <v>GLUKtoFZUK</v>
+      </c>
+      <c r="B70" s="51" t="str">
+        <f t="shared" ref="B70:B73" si="42">MID(A70,1,SEARCH("to",A70)-1)</f>
+        <v>GLUK</v>
+      </c>
+      <c r="C70" s="51" t="str">
+        <f t="shared" ref="C70:C73" si="43">MID(A70,SEARCH("to",A70)+2,99)</f>
+        <v>FZUK</v>
+      </c>
+      <c r="D70" s="97" t="s">
+        <v>262</v>
+      </c>
+      <c r="E70" s="99"/>
+      <c r="F70" s="36">
+        <f t="shared" si="7"/>
+        <v>160</v>
+      </c>
+      <c r="G70" s="38">
+        <f>IF(M70="multiply",F70,F71)</f>
+        <v>160</v>
+      </c>
+      <c r="H70" s="9">
+        <f t="shared" si="33"/>
+        <v>4546.09</v>
+      </c>
+      <c r="I70" s="9">
+        <f t="shared" si="27"/>
+        <v>28.413062500000002</v>
+      </c>
+      <c r="J70" t="str">
+        <f t="shared" si="28"/>
+        <v>GlukFzuk</v>
+      </c>
+      <c r="K70" t="str">
+        <f t="shared" si="29"/>
+        <v>constFactorGlukFzuk</v>
+      </c>
+      <c r="M70" s="38" t="str">
+        <f>IF(H70&gt;I70,"multiply","  divide")</f>
+        <v>multiply</v>
+      </c>
+      <c r="N70" s="38" t="str">
+        <f>IF(M70="multiply",PROPER(B70)&amp;PROPER(C70),J71)</f>
+        <v>GlukFzuk</v>
+      </c>
+    </row>
+    <row r="71" spans="1:14" ht="18">
+      <c r="A71" s="50" t="str">
+        <f t="shared" si="30"/>
+        <v>FZUKtoGLUK</v>
+      </c>
+      <c r="B71" s="51" t="str">
+        <f t="shared" si="42"/>
+        <v>FZUK</v>
+      </c>
+      <c r="C71" s="51" t="str">
+        <f t="shared" si="43"/>
+        <v>GLUK</v>
+      </c>
+      <c r="D71" s="97" t="s">
+        <v>263</v>
+      </c>
+      <c r="E71" s="48"/>
+      <c r="F71" s="36">
+        <f t="shared" si="7"/>
+        <v>6.2500000000000003E-3</v>
+      </c>
+      <c r="G71" s="38">
+        <f>IF(M71="multiply",F71,F70)</f>
+        <v>160</v>
+      </c>
+      <c r="H71" s="9">
+        <f t="shared" si="33"/>
+        <v>28.413062500000002</v>
+      </c>
+      <c r="I71" s="9">
+        <f t="shared" si="27"/>
+        <v>4546.09</v>
+      </c>
+      <c r="J71" t="str">
+        <f t="shared" si="28"/>
+        <v>FzukGluk</v>
+      </c>
+      <c r="K71" t="str">
+        <f t="shared" si="29"/>
+        <v>constFactorFzukGluk</v>
+      </c>
+      <c r="M71" s="38" t="str">
+        <f>IF(M70="multiply","  divide","multiply")</f>
+        <v xml:space="preserve">  divide</v>
+      </c>
+      <c r="N71" s="38" t="str">
+        <f>IF(M71="multiply",PROPER(B71)&amp;PROPER(C71),J70)</f>
+        <v>GlukFzuk</v>
+      </c>
+    </row>
+    <row r="72" spans="1:14" ht="18">
+      <c r="A72" s="50" t="str">
+        <f t="shared" si="30"/>
+        <v>GLUStoFZUS</v>
+      </c>
+      <c r="B72" s="51" t="str">
+        <f t="shared" si="42"/>
+        <v>GLUS</v>
+      </c>
+      <c r="C72" s="51" t="str">
+        <f t="shared" si="43"/>
+        <v>FZUS</v>
+      </c>
+      <c r="D72" s="97" t="s">
+        <v>264</v>
+      </c>
+      <c r="E72" s="48"/>
+      <c r="F72" s="36">
+        <f t="shared" si="7"/>
+        <v>128</v>
+      </c>
+      <c r="G72" s="39">
+        <f>IF(M72="multiply",F72,F73)</f>
+        <v>128</v>
+      </c>
+      <c r="H72" s="9">
+        <f t="shared" si="33"/>
+        <v>3785.4117839999999</v>
+      </c>
+      <c r="I72" s="9">
+        <f t="shared" si="27"/>
+        <v>29.573529562499999</v>
+      </c>
+      <c r="J72" t="str">
+        <f t="shared" si="28"/>
+        <v>GlusFzus</v>
+      </c>
+      <c r="K72" t="str">
+        <f t="shared" si="29"/>
+        <v>constFactorGlusFzus</v>
+      </c>
+      <c r="M72" s="39" t="str">
+        <f>IF(H72&gt;I72,"multiply","  divide")</f>
+        <v>multiply</v>
+      </c>
+      <c r="N72" s="39" t="str">
+        <f>IF(M72="multiply",PROPER(B72)&amp;PROPER(C72),J73)</f>
+        <v>GlusFzus</v>
+      </c>
+    </row>
+    <row r="73" spans="1:14" ht="19" thickBot="1">
+      <c r="A73" s="50" t="str">
+        <f t="shared" si="30"/>
+        <v>FZUStoGLUS</v>
+      </c>
+      <c r="B73" s="51" t="str">
+        <f t="shared" si="42"/>
+        <v>FZUS</v>
+      </c>
+      <c r="C73" s="51" t="str">
+        <f t="shared" si="43"/>
+        <v>GLUS</v>
+      </c>
+      <c r="D73" s="98" t="s">
+        <v>265</v>
+      </c>
+      <c r="E73" s="49"/>
+      <c r="F73" s="36">
+        <f t="shared" si="7"/>
+        <v>7.8125E-3</v>
+      </c>
+      <c r="G73" s="39">
+        <f>IF(M73="multiply",F73,F72)</f>
+        <v>128</v>
+      </c>
+      <c r="H73" s="9">
+        <f t="shared" si="33"/>
+        <v>29.573529562499999</v>
+      </c>
+      <c r="I73" s="9">
+        <f t="shared" si="27"/>
+        <v>3785.4117839999999</v>
+      </c>
+      <c r="J73" t="str">
+        <f t="shared" si="28"/>
+        <v>FzusGlus</v>
+      </c>
+      <c r="K73" t="str">
+        <f t="shared" si="29"/>
+        <v>constFactorFzusGlus</v>
+      </c>
+      <c r="M73" s="39" t="str">
+        <f>IF(M72="multiply","  divide","multiply")</f>
+        <v xml:space="preserve">  divide</v>
+      </c>
+      <c r="N73" s="39" t="str">
+        <f>IF(M73="multiply",PROPER(B73)&amp;PROPER(C73),J72)</f>
+        <v>GlusFzus</v>
       </c>
     </row>
   </sheetData>
@@ -6931,17 +7383,17 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:2">
-      <c r="B2" s="65" t="s">
+      <c r="B2" s="64" t="s">
         <v>220</v>
       </c>
     </row>
     <row r="3" spans="2:2" ht="46">
-      <c r="B3" s="64" t="s">
+      <c r="B3" s="63" t="s">
         <v>219</v>
       </c>
     </row>
     <row r="4" spans="2:2" ht="46">
-      <c r="B4" s="64" t="s">
+      <c r="B4" s="63" t="s">
         <v>221</v>
       </c>
     </row>
@@ -6951,12 +7403,12 @@
       </c>
     </row>
     <row r="9" spans="2:2">
-      <c r="B9" s="66" t="s">
+      <c r="B9" s="65" t="s">
         <v>222</v>
       </c>
     </row>
     <row r="12" spans="2:2" ht="20">
-      <c r="B12" s="57" t="s">
+      <c r="B12" s="56" t="s">
         <v>212</v>
       </c>
     </row>
@@ -6981,7 +7433,7 @@
       </c>
     </row>
     <row r="19" spans="2:2" ht="51">
-      <c r="B19" s="67" t="s">
+      <c r="B19" s="66" t="s">
         <v>224</v>
       </c>
     </row>
@@ -7005,43 +7457,43 @@
   </cols>
   <sheetData>
     <row r="1" spans="3:4">
-      <c r="C1" s="68" t="s">
+      <c r="C1" s="67" t="s">
         <v>237</v>
       </c>
     </row>
     <row r="4" spans="3:4">
-      <c r="C4" s="66" t="s">
+      <c r="C4" s="65" t="s">
         <v>233</v>
       </c>
     </row>
     <row r="5" spans="3:4">
-      <c r="C5" s="66" t="s">
+      <c r="C5" s="65" t="s">
         <v>234</v>
       </c>
     </row>
     <row r="8" spans="3:4">
-      <c r="C8" s="66" t="s">
+      <c r="C8" s="65" t="s">
         <v>238</v>
       </c>
-      <c r="D8" s="68" t="s">
+      <c r="D8" s="67" t="s">
         <v>239</v>
       </c>
     </row>
     <row r="9" spans="3:4">
-      <c r="C9" s="66" t="s">
+      <c r="C9" s="65" t="s">
         <v>235</v>
       </c>
-      <c r="D9" s="66" t="s">
+      <c r="D9" s="65" t="s">
         <v>236</v>
       </c>
     </row>
     <row r="12" spans="3:4">
-      <c r="C12" s="68" t="s">
+      <c r="C12" s="67" t="s">
         <v>244</v>
       </c>
     </row>
     <row r="13" spans="3:4" ht="119">
-      <c r="C13" s="63" t="s">
+      <c r="C13" s="62" t="s">
         <v>243</v>
       </c>
     </row>
@@ -7051,17 +7503,17 @@
       </c>
     </row>
     <row r="16" spans="3:4">
-      <c r="C16" s="66" t="s">
+      <c r="C16" s="65" t="s">
         <v>245</v>
       </c>
     </row>
     <row r="18" spans="3:3">
-      <c r="C18" s="68" t="s">
+      <c r="C18" s="67" t="s">
         <v>250</v>
       </c>
     </row>
     <row r="19" spans="3:3">
-      <c r="C19" s="66" t="s">
+      <c r="C19" s="65" t="s">
         <v>251</v>
       </c>
     </row>
@@ -7072,7 +7524,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{12AF49E5-C5CF-EF45-BD21-7588D88F54A2}">
-  <dimension ref="A1:C43"/>
+  <dimension ref="A1:C47"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="18" bestFit="1" customWidth="1"/>
@@ -7431,6 +7883,38 @@
         <v>200</v>
       </c>
     </row>
+    <row r="44" spans="1:3">
+      <c r="A44" s="100" t="s">
+        <v>262</v>
+      </c>
+      <c r="B44" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3">
+      <c r="A45" s="100" t="s">
+        <v>263</v>
+      </c>
+      <c r="B45" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3">
+      <c r="A46" s="100" t="s">
+        <v>264</v>
+      </c>
+      <c r="B46" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3">
+      <c r="A47" s="100" t="s">
+        <v>265</v>
+      </c>
+      <c r="B47" t="s">
+        <v>269</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>